<commit_message>
feat(pipeline): implement translation service and update schemas
Add translation service modules and update JSON schemas for stress
and test data. This also includes adding markdown and beautifulsoup4
to requirements.txt and cleaning up temporary excel reports.
</commit_message>
<xml_diff>
--- a/Hybrid_test_report.xlsx
+++ b/Hybrid_test_report.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>21.166 ms</t>
+          <t>79.617 ms</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="I5" s="10" t="n">
-        <v>32.63810000498779</v>
+        <v>121918.2281999965</v>
       </c>
       <c r="J5" s="10" t="inlineStr">
         <is>
@@ -1083,9 +1083,9 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t># Projektname: Globale Kundenmanagement-Plattform (GKMP)
-## Projektübersicht
-Die Globale Kundenmanagement-Plattform (GKMP) stellt eine zentrale Lösung für die Verwaltung von Kundeninformationen über verschiedene Regionen, Geschäftsbereiche und regulatorische Zuständigkeiten hinweg bereit.</t>
+          <t>Projektname: Globale Kundenmanagement-Plattform (GKMP) 
+ Projektübersicht 
+ Die Globale Kundenmanagement-Plattform (GKMP) stellt eine zentrale Lösung für die Verwaltung von Kundeninformationen über verschiedene Regionen, Geschäftsbereiche und regulatorische Zuständigkeiten hinweg bereit.</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -1095,14 +1095,14 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.9413</t>
+          <t>fasttext/0.9483</t>
         </is>
       </c>
       <c r="F5" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="6">
@@ -1130,10 +1130,10 @@
         </is>
       </c>
       <c r="F6" s="12" t="n">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>435</v>
+        <v>432</v>
       </c>
     </row>
     <row r="7">
@@ -1148,7 +1148,7 @@
       <c r="C7" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-Die Lösung unterstützt deutschsprachige und englischsprachige Benutzer und ermöglicht eine nahtlose Integration mit bestehenden Unternehmensanwendungen.</t>
+ Die Lösung unterstützt deutschsprachige und englischsprachige Benutzer und ermöglicht eine nahtlose Integration mit bestehenden Unternehmensanwendungen.</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -1162,10 +1162,10 @@
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>589</v>
+        <v>587</v>
       </c>
     </row>
     <row r="8">
@@ -1193,10 +1193,10 @@
         </is>
       </c>
       <c r="F8" s="12" t="n">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>785</v>
+        <v>783</v>
       </c>
     </row>
     <row r="9">
@@ -1211,7 +1211,7 @@
       <c r="C9" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-Das System muss hochverfügbar sein und eine Verarbeitung großer Datenmengen mit minimaler Latenz gewährleisten.</t>
+ Das System muss hochverfügbar sein und eine Verarbeitung großer Datenmengen mit minimaler Latenz gewährleisten.</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
@@ -1225,10 +1225,10 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="10">
@@ -1256,10 +1256,10 @@
         </is>
       </c>
       <c r="F10" s="12" t="n">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="11">
@@ -1274,9 +1274,8 @@
       <c r="C11" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# Geschäftlicher Hintergrund
-Das Unternehmen betreibt derzeit mehrere voneinander unabhängige Anwendungen zur Speicherung von Kundendaten.</t>
+ Geschäftlicher Hintergrund 
+ Das Unternehmen betreibt derzeit mehrere voneinander unabhängige Anwendungen zur Speicherung von Kundendaten.</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -1286,14 +1285,14 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.9497</t>
+          <t>fasttext/0.9752</t>
         </is>
       </c>
       <c r="F11" s="9" t="n">
         <v>1022</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>1168</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="12">
@@ -1321,10 +1320,10 @@
         </is>
       </c>
       <c r="F12" s="12" t="n">
-        <v>1169</v>
+        <v>1165</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>1288</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="13">
@@ -1339,7 +1338,7 @@
       <c r="C13" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-The new platform aims to establish a single source of truth for customer information and improve operational efficiency across departments.</t>
+ The new platform aims to establish a single source of truth for customer information and improve operational efficiency across departments.</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
@@ -1353,10 +1352,10 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>1288</v>
+        <v>1285</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>1429</v>
+        <v>1426</v>
       </c>
     </row>
     <row r="14">
@@ -1371,7 +1370,7 @@
       <c r="C14" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-Mehrere Fachabteilungen haben Bedenken hinsichtlich Datenqualität, Berichtsverzögerungen und regulatorischer Compliance geäußert.</t>
+ Mehrere Fachabteilungen haben Bedenken hinsichtlich Datenqualität, Berichtsverzögerungen und regulatorischer Compliance geäußert.</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
@@ -1385,10 +1384,10 @@
         </is>
       </c>
       <c r="F14" s="12" t="n">
-        <v>1429</v>
+        <v>1427</v>
       </c>
       <c r="G14" s="13" t="n">
-        <v>1560</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="15">
@@ -1416,10 +1415,10 @@
         </is>
       </c>
       <c r="F15" s="9" t="n">
-        <v>1561</v>
+        <v>1559</v>
       </c>
       <c r="G15" s="10" t="n">
-        <v>1713</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="16">
@@ -1434,25 +1433,23 @@
       <c r="C16" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# Geschäftsziele
-## Primäre Ziele
-* Zentralisierung sämtlicher Kundendaten
-* Verbesserung der Datenqualität
-* Reduzierung redundanter Datensätze
-* Einhaltung regulatorischer Anforderungen
-* Unterstützung internationaler Geschäftsprozesse
-* Verbesserung der Such- und Analysefunktionen
-## Secondary Objectives
-* Faster customer onboarding
-* Improved reporting capabilities
-* Enhanced audit traceability
-* Better integration with third-party systems
-* Reduced operational overhead
----
-# Benutzerrollen
-## Vertriebssachbearbeiter
-Der Vertriebssachbearbeiter verwaltet Kundenprofile, erstellt Verträge und pflegt Stammdaten.</t>
+ Geschäftsziele 
+ Primäre Ziele 
+ Zentralisierung sämtlicher Kundendaten 
+ Verbesserung der Datenqualität 
+ Reduzierung redundanter Datensätze 
+ Einhaltung regulatorischer Anforderungen 
+ Unterstützung internationaler Geschäftsprozesse 
+ Verbesserung der Such- und Analysefunktionen 
+ Secondary Objectives 
+ Faster customer onboarding 
+ Improved reporting capabilities 
+ Enhanced audit traceability 
+ Better integration with third-party systems 
+ Reduced operational overhead 
+ Benutzerrollen 
+ Vertriebssachbearbeiter 
+ Der Vertriebssachbearbeiter verwaltet Kundenprofile, erstellt Verträge und pflegt Stammdaten.</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
@@ -1462,14 +1459,14 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.8633</t>
+          <t>fasttext/0.9065</t>
         </is>
       </c>
       <c r="F16" s="12" t="n">
-        <v>1713</v>
+        <v>1712</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>2348</v>
+        <v>2339</v>
       </c>
     </row>
     <row r="17">
@@ -1484,8 +1481,8 @@
       <c r="C17" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Kundendienstmitarbeiter
-Customer Service Representatives assist customers, update customer information, and resolve support requests.</t>
+ Kundendienstmitarbeiter 
+ Customer Service Representatives assist customers, update customer information, and resolve support requests.</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -1495,14 +1492,14 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.5390</t>
+          <t>fasttext/0.5710</t>
         </is>
       </c>
       <c r="F17" s="9" t="n">
-        <v>2348</v>
+        <v>2340</v>
       </c>
       <c r="G17" s="10" t="n">
-        <v>2487</v>
+        <v>2477</v>
       </c>
     </row>
     <row r="18">
@@ -1517,8 +1514,8 @@
       <c r="C18" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Compliance-Beauftragter
-Der Compliance-Beauftragte überwacht regulatorische Anforderungen und prüft Einwilligungsnachweise.</t>
+ Compliance-Beauftragter 
+ Der Compliance-Beauftragte überwacht regulatorische Anforderungen und prüft Einwilligungsnachweise.</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
@@ -1528,14 +1525,14 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.9822</t>
+          <t>fasttext/0.9872</t>
         </is>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2487</v>
+        <v>2478</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>2616</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="19">
@@ -1550,8 +1547,8 @@
       <c r="C19" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Systemadministrator
-System Administrators manage configurations, user access, monitoring, and platform maintenance.</t>
+ Systemadministrator 
+ System Administrators manage configurations, user access, monitoring, and platform maintenance.</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
@@ -1561,14 +1558,14 @@
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.6972</t>
+          <t>fasttext/0.7561</t>
         </is>
       </c>
       <c r="F19" s="9" t="n">
-        <v>2616</v>
+        <v>2606</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>2737</v>
+        <v>2725</v>
       </c>
     </row>
     <row r="20">
@@ -1583,8 +1580,8 @@
       <c r="C20" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Berichtsanalyst
-Reporting Analysts generate operational, financial, and compliance reports.</t>
+ Berichtsanalyst 
+ Reporting Analysts generate operational, financial, and compliance reports.</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
@@ -1594,14 +1591,14 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.7126</t>
+          <t>fasttext/0.7651</t>
         </is>
       </c>
       <c r="F20" s="12" t="n">
-        <v>2737</v>
+        <v>2726</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>2834</v>
+        <v>2821</v>
       </c>
     </row>
     <row r="21">
@@ -1616,10 +1613,9 @@
       <c r="C21" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# User Story US-001 – Kundensuche
-## Beschreibung
-Als Kundendienstmitarbeiter möchte ich Kunden anhand verschiedener Suchkriterien finden können, damit ich Kundeninformationen schnell abrufen kann.</t>
+ User Story US-001 – Kundensuche 
+ Beschreibung 
+ Als Kundendienstmitarbeiter möchte ich Kunden anhand verschiedener Suchkriterien finden können, damit ich Kundeninformationen schnell abrufen kann.</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
@@ -1629,14 +1625,14 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.8382</t>
+          <t>fasttext/0.8958</t>
         </is>
       </c>
       <c r="F21" s="9" t="n">
-        <v>2834</v>
+        <v>2822</v>
       </c>
       <c r="G21" s="10" t="n">
-        <v>3040</v>
+        <v>3022</v>
       </c>
     </row>
     <row r="22">
@@ -1651,7 +1647,7 @@
       <c r="C22" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-The system shall provide advanced search capabilities supporting exact and fuzzy matching.</t>
+ The system shall provide advanced search capabilities supporting exact and fuzzy matching.</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
@@ -1665,10 +1661,10 @@
         </is>
       </c>
       <c r="F22" s="12" t="n">
-        <v>3040</v>
+        <v>3023</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>3132</v>
+        <v>3115</v>
       </c>
     </row>
     <row r="23">
@@ -1683,18 +1679,18 @@
       <c r="C23" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Suchkriterien
-Der Benutzer soll Kunden anhand folgender Felder suchen können:
-* Kundennummer
-* Vorname
-* Nachname
-* E-Mail-Adresse
-* Telefonnummer
-* Geburtsdatum
-* Vertragsnummer
-* Kundenstatus
-## Akzeptanzkriterien
-* Das Feld "Kundennummer" muss durchsuchbar sein.</t>
+ Suchkriterien 
+ Der Benutzer soll Kunden anhand folgender Felder suchen können: 
+ Kundennummer 
+ Vorname 
+ Nachname 
+ E-Mail-Adresse 
+ Telefonnummer 
+ Geburtsdatum 
+ Vertragsnummer 
+ Kundenstatus 
+ Akzeptanzkriterien 
+ Das Feld "Kundennummer" muss durchsuchbar sein.</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
@@ -1704,14 +1700,14 @@
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.9609</t>
+          <t>fasttext/0.9732</t>
         </is>
       </c>
       <c r="F23" s="9" t="n">
-        <v>3132</v>
+        <v>3116</v>
       </c>
       <c r="G23" s="10" t="n">
-        <v>3406</v>
+        <v>3390</v>
       </c>
     </row>
     <row r="24">
@@ -1726,7 +1722,7 @@
       <c r="C24" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Das Feld "Nachname" muss unterstützt werden.</t>
+ Das Feld "Nachname" muss unterstützt werden.</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -1740,10 +1736,10 @@
         </is>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3406</v>
+        <v>3391</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>3453</v>
+        <v>3437</v>
       </c>
     </row>
     <row r="25">
@@ -1758,7 +1754,7 @@
       <c r="C25" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Das Feld "Vorname" muss unterstützt werden.</t>
+ Das Feld "Vorname" muss unterstützt werden.</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
@@ -1772,10 +1768,10 @@
         </is>
       </c>
       <c r="F25" s="9" t="n">
-        <v>3453</v>
+        <v>3438</v>
       </c>
       <c r="G25" s="10" t="n">
-        <v>3499</v>
+        <v>3483</v>
       </c>
     </row>
     <row r="26">
@@ -1790,7 +1786,7 @@
       <c r="C26" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Search results shall be returned within three seconds.</t>
+ Search results shall be returned within three seconds.</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -1804,10 +1800,10 @@
         </is>
       </c>
       <c r="F26" s="12" t="n">
-        <v>3499</v>
+        <v>3484</v>
       </c>
       <c r="G26" s="13" t="n">
-        <v>3556</v>
+        <v>3540</v>
       </c>
     </row>
     <row r="27">
@@ -1822,7 +1818,7 @@
       <c r="C27" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Die Trefferliste muss paginiert dargestellt werden.</t>
+ Die Trefferliste muss paginiert dargestellt werden.</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
@@ -1836,10 +1832,10 @@
         </is>
       </c>
       <c r="F27" s="9" t="n">
-        <v>3556</v>
+        <v>3541</v>
       </c>
       <c r="G27" s="10" t="n">
-        <v>3610</v>
+        <v>3594</v>
       </c>
     </row>
     <row r="28">
@@ -1854,7 +1850,7 @@
       <c r="C28" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* The system shall support fuzzy search functionality.</t>
+ The system shall support fuzzy search functionality.</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1868,10 +1864,10 @@
         </is>
       </c>
       <c r="F28" s="12" t="n">
-        <v>3610</v>
+        <v>3595</v>
       </c>
       <c r="G28" s="13" t="n">
-        <v>3665</v>
+        <v>3649</v>
       </c>
     </row>
     <row r="29">
@@ -1886,7 +1882,7 @@
       <c r="C29" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Die Suche muss Groß- und Kleinschreibung ignorieren.</t>
+ Die Suche muss Groß- und Kleinschreibung ignorieren.</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
@@ -1900,10 +1896,10 @@
         </is>
       </c>
       <c r="F29" s="9" t="n">
-        <v>3665</v>
+        <v>3650</v>
       </c>
       <c r="G29" s="10" t="n">
-        <v>3720</v>
+        <v>3704</v>
       </c>
     </row>
     <row r="30">
@@ -1918,7 +1914,7 @@
       <c r="C30" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Search filters shall support multiple simultaneous criteria.</t>
+ Search filters shall support multiple simultaneous criteria.</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1932,10 +1928,10 @@
         </is>
       </c>
       <c r="F30" s="12" t="n">
-        <v>3720</v>
+        <v>3705</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>3783</v>
+        <v>3767</v>
       </c>
     </row>
     <row r="31">
@@ -1950,7 +1946,7 @@
       <c r="C31" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Suchergebnisse müssen nach Relevanz sortiert werden können.</t>
+ Suchergebnisse müssen nach Relevanz sortiert werden können.</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
@@ -1964,10 +1960,10 @@
         </is>
       </c>
       <c r="F31" s="9" t="n">
-        <v>3783</v>
+        <v>3768</v>
       </c>
       <c r="G31" s="10" t="n">
-        <v>3845</v>
+        <v>3829</v>
       </c>
     </row>
     <row r="32">
@@ -1982,10 +1978,9 @@
       <c r="C32" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# User Story US-002 – Einwilligungsverwaltung
-## Beschreibung
-Als Compliance-Beauftragter möchte ich sämtliche Kundeneinwilligungen einsehen können, damit regulatorische Anforderungen überprüft werden können.</t>
+ User Story US-002 – Einwilligungsverwaltung 
+ Beschreibung 
+ Als Compliance-Beauftragter möchte ich sämtliche Kundeneinwilligungen einsehen können, damit regulatorische Anforderungen überprüft werden können.</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -1995,14 +1990,14 @@
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.9718</t>
+          <t>fasttext/0.9839</t>
         </is>
       </c>
       <c r="F32" s="12" t="n">
-        <v>3845</v>
+        <v>3830</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>4062</v>
+        <v>4043</v>
       </c>
     </row>
     <row r="33">
@@ -2017,14 +2012,14 @@
       <c r="C33" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Funktionale Anforderungen
-Der Compliance-Beauftragte muss folgende Informationen anzeigen können:
-* Einwilligungsstatus
-* Zeitstempel
-* Herkunftssystem
-* Änderungsverlauf
-* Verantwortlicher Benutzer
-The system shall preserve historical records for auditing purposes.</t>
+ Funktionale Anforderungen 
+ Der Compliance-Beauftragte muss folgende Informationen anzeigen können: 
+ Einwilligungsstatus 
+ Zeitstempel 
+ Herkunftssystem 
+ Änderungsverlauf 
+ Verantwortlicher Benutzer 
+ The system shall preserve historical records for auditing purposes.</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
@@ -2034,14 +2029,14 @@
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.9597</t>
+          <t>fasttext/0.9649</t>
         </is>
       </c>
       <c r="F33" s="9" t="n">
-        <v>4062</v>
+        <v>4044</v>
       </c>
       <c r="G33" s="10" t="n">
-        <v>4336</v>
+        <v>4320</v>
       </c>
     </row>
     <row r="34">
@@ -2056,8 +2051,8 @@
       <c r="C34" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Akzeptanzkriterien
-* Einwilligungshistorien dürfen nicht bearbeitet werden.</t>
+ Akzeptanzkriterien 
+ Einwilligungshistorien dürfen nicht bearbeitet werden.</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -2067,14 +2062,14 @@
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.9764</t>
+          <t>fasttext/0.9848</t>
         </is>
       </c>
       <c r="F34" s="12" t="n">
-        <v>4336</v>
+        <v>4321</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>4417</v>
+        <v>4400</v>
       </c>
     </row>
     <row r="35">
@@ -2089,7 +2084,7 @@
       <c r="C35" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Änderungen müssen revisionssicher gespeichert werden.</t>
+ Änderungen müssen revisionssicher gespeichert werden.</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
@@ -2103,10 +2098,10 @@
         </is>
       </c>
       <c r="F35" s="9" t="n">
-        <v>4417</v>
+        <v>4401</v>
       </c>
       <c r="G35" s="10" t="n">
-        <v>4473</v>
+        <v>4456</v>
       </c>
     </row>
     <row r="36">
@@ -2121,7 +2116,7 @@
       <c r="C36" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Auditberichte müssen als PDF und Excel exportierbar sein.</t>
+ Auditberichte müssen als PDF und Excel exportierbar sein.</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -2135,10 +2130,10 @@
         </is>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4473</v>
+        <v>4457</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>4533</v>
+        <v>4516</v>
       </c>
     </row>
     <row r="37">
@@ -2153,7 +2148,7 @@
       <c r="C37" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Das System muss sämtliche Zugriffe protokollieren.</t>
+ Das System muss sämtliche Zugriffe protokollieren.</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
@@ -2167,10 +2162,10 @@
         </is>
       </c>
       <c r="F37" s="9" t="n">
-        <v>4533</v>
+        <v>4517</v>
       </c>
       <c r="G37" s="10" t="n">
-        <v>4586</v>
+        <v>4569</v>
       </c>
     </row>
     <row r="38">
@@ -2185,7 +2180,7 @@
       <c r="C38" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Historical records shall remain available indefinitely.</t>
+ Historical records shall remain available indefinitely.</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -2199,10 +2194,10 @@
         </is>
       </c>
       <c r="F38" s="12" t="n">
-        <v>4586</v>
+        <v>4570</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>4644</v>
+        <v>4627</v>
       </c>
     </row>
     <row r="39">
@@ -2217,7 +2212,7 @@
       <c r="C39" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Jede Änderung muss einem Benutzer zugeordnet werden können.</t>
+ Jede Änderung muss einem Benutzer zugeordnet werden können.</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
@@ -2231,10 +2226,10 @@
         </is>
       </c>
       <c r="F39" s="9" t="n">
-        <v>4644</v>
+        <v>4628</v>
       </c>
       <c r="G39" s="10" t="n">
-        <v>4706</v>
+        <v>4689</v>
       </c>
     </row>
     <row r="40">
@@ -2249,10 +2244,9 @@
       <c r="C40" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# Technische Architektur
-## Architekturübersicht
-The application follows a microservice architecture consisting of independently deployable services.</t>
+ Technische Architektur 
+ Architekturübersicht 
+ The application follows a microservice architecture consisting of independently deployable services.</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -2262,14 +2256,14 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.3368</t>
+          <t>fasttext/0.4312</t>
         </is>
       </c>
       <c r="F40" s="12" t="n">
-        <v>4706</v>
+        <v>4690</v>
       </c>
       <c r="G40" s="13" t="n">
-        <v>4864</v>
+        <v>4844</v>
       </c>
     </row>
     <row r="41">
@@ -2284,7 +2278,7 @@
       <c r="C41" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-Jeder Service besitzt eine klar definierte Verantwortlichkeit und kommuniziert über standardisierte REST-Schnittstellen.</t>
+ Jeder Service besitzt eine klar definierte Verantwortlichkeit und kommuniziert über standardisierte REST-Schnittstellen.</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -2298,10 +2292,10 @@
         </is>
       </c>
       <c r="F41" s="9" t="n">
-        <v>4864</v>
+        <v>4845</v>
       </c>
       <c r="G41" s="10" t="n">
-        <v>4986</v>
+        <v>4967</v>
       </c>
     </row>
     <row r="42">
@@ -2316,8 +2310,8 @@
       <c r="C42" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## API-Gateway
-Das API-Gateway fungiert als zentraler Einstiegspunkt für sämtliche Client-Anfragen.</t>
+ API-Gateway 
+ Das API-Gateway fungiert als zentraler Einstiegspunkt für sämtliche Client-Anfragen.</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -2327,14 +2321,14 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.9510</t>
+          <t>fasttext/0.9620</t>
         </is>
       </c>
       <c r="F42" s="12" t="n">
-        <v>4986</v>
+        <v>4968</v>
       </c>
       <c r="G42" s="13" t="n">
-        <v>5088</v>
+        <v>5068</v>
       </c>
     </row>
     <row r="43">
@@ -2349,18 +2343,18 @@
       <c r="C43" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-Funktionen:
-* Authentifizierung
-* Autorisierung
-* Routing
-* Lastverteilung
-* API-Protokollierung
-## Authentifizierung
-Die Authentifizierung erfolgt über:
-* OAuth 2.0
-* OpenID Connect
-* Multi-Faktor-Authentifizierung
-The system shall support integration with enterprise identity providers.</t>
+ Funktionen: 
+ Authentifizierung 
+ Autorisierung 
+ Routing 
+ Lastverteilung 
+ API-Protokollierung 
+ Authentifizierung 
+ Die Authentifizierung erfolgt über: 
+ OAuth 2.0 
+ OpenID Connect 
+ Multi-Faktor-Authentifizierung 
+ The system shall support integration with enterprise identity providers.</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
@@ -2370,14 +2364,14 @@
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.8696</t>
+          <t>fasttext/0.8792</t>
         </is>
       </c>
       <c r="F43" s="9" t="n">
-        <v>5088</v>
+        <v>5069</v>
       </c>
       <c r="G43" s="10" t="n">
-        <v>5383</v>
+        <v>5370</v>
       </c>
     </row>
     <row r="44">
@@ -2392,10 +2386,9 @@
       <c r="C44" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# Kerndienste
-## Kundenservice
-Verwaltung von Kundenstammdaten und Kundenbeziehungen.</t>
+ Kerndienste 
+ Kundenservice 
+ Verwaltung von Kundenstammdaten und Kundenbeziehungen.</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -2405,14 +2398,14 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.6938</t>
+          <t>fasttext/0.8646</t>
         </is>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5383</v>
+        <v>5371</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>5477</v>
+        <v>5459</v>
       </c>
     </row>
     <row r="45">
@@ -2427,8 +2420,8 @@
       <c r="C45" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Vertragsservice
-Verwaltung sämtlicher Vertragsinformationen.</t>
+ Vertragsservice 
+ Verwaltung sämtlicher Vertragsinformationen.</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
@@ -2438,14 +2431,14 @@
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.8163</t>
+          <t>fasttext/0.8699</t>
         </is>
       </c>
       <c r="F45" s="9" t="n">
-        <v>5477</v>
+        <v>5460</v>
       </c>
       <c r="G45" s="10" t="n">
-        <v>5543</v>
+        <v>5524</v>
       </c>
     </row>
     <row r="46">
@@ -2460,8 +2453,8 @@
       <c r="C46" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Benachrichtigungsservice
-Versand von E-Mails, SMS-Nachrichten und Systembenachrichtigungen.</t>
+ Benachrichtigungsservice 
+ Versand von E-Mails, SMS-Nachrichten und Systembenachrichtigungen.</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -2471,14 +2464,14 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.8930</t>
+          <t>fasttext/0.9218</t>
         </is>
       </c>
       <c r="F46" s="12" t="n">
-        <v>5543</v>
+        <v>5525</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>5640</v>
+        <v>5620</v>
       </c>
     </row>
     <row r="47">
@@ -2493,8 +2486,8 @@
       <c r="C47" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Audit-Service
-Speicherung aller revisionsrelevanten Ereignisse.</t>
+ Audit-Service 
+ Speicherung aller revisionsrelevanten Ereignisse.</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
@@ -2504,14 +2497,14 @@
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.4024</t>
+          <t>fasttext/0.5014</t>
         </is>
       </c>
       <c r="F47" s="9" t="n">
-        <v>5640</v>
+        <v>5621</v>
       </c>
       <c r="G47" s="10" t="n">
-        <v>5709</v>
+        <v>5688</v>
       </c>
     </row>
     <row r="48">
@@ -2526,8 +2519,8 @@
       <c r="C48" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Berichtsservice
-Generierung operativer und regulatorischer Berichte.</t>
+ Berichtsservice 
+ Generierung operativer und regulatorischer Berichte.</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -2537,14 +2530,14 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.8699</t>
+          <t>fasttext/0.9037</t>
         </is>
       </c>
       <c r="F48" s="12" t="n">
-        <v>5709</v>
+        <v>5689</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>5783</v>
+        <v>5761</v>
       </c>
     </row>
     <row r="49">
@@ -2559,8 +2552,8 @@
       <c r="C49" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Integrationsservice
-The Integration Service shall synchronize information with external systems.</t>
+ Integrationsservice 
+ The Integration Service shall synchronize information with external systems.</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
@@ -2570,14 +2563,14 @@
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.7223</t>
+          <t>fasttext/0.7880</t>
         </is>
       </c>
       <c r="F49" s="9" t="n">
-        <v>5783</v>
+        <v>5762</v>
       </c>
       <c r="G49" s="10" t="n">
-        <v>5885</v>
+        <v>5862</v>
       </c>
     </row>
     <row r="50">
@@ -2592,8 +2585,8 @@
       <c r="C50" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Compliance-Service
-Der Compliance-Service überwacht regulatorische Anforderungen und Datenschutzrichtlinien.</t>
+ Compliance-Service 
+ Der Compliance-Service überwacht regulatorische Anforderungen und Datenschutzrichtlinien.</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -2603,14 +2596,14 @@
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.9181</t>
+          <t>fasttext/0.9397</t>
         </is>
       </c>
       <c r="F50" s="12" t="n">
-        <v>5885</v>
+        <v>5863</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>5999</v>
+        <v>5975</v>
       </c>
     </row>
     <row r="51">
@@ -2625,9 +2618,8 @@
       <c r="C51" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# Ereignisgesteuerte Kommunikation
-Die Plattform verwendet Apache Kafka für die asynchrone Kommunikation zwischen Services.</t>
+ Ereignisgesteuerte Kommunikation 
+ Die Plattform verwendet Apache Kafka für die asynchrone Kommunikation zwischen Services.</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
@@ -2637,14 +2629,14 @@
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.8195</t>
+          <t>fasttext/0.8965</t>
         </is>
       </c>
       <c r="F51" s="9" t="n">
-        <v>5999</v>
+        <v>5976</v>
       </c>
       <c r="G51" s="10" t="n">
-        <v>6130</v>
+        <v>6103</v>
       </c>
     </row>
     <row r="52">
@@ -2659,17 +2651,16 @@
       <c r="C52" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-Examples of business events:
-* KundeErstellt
-* KundeAktualisiert
-* VertragAngelegt
-* EinwilligungErteilt
-* EinwilligungWiderrufen
----
-# Datenbankanforderungen
-## Kundentabelle
-Die Kundendatenbank muss folgende Felder unterstützen:
-| Feldname                    |
+ Examples of business events: 
+ KundeErstellt 
+ KundeAktualisiert 
+ VertragAngelegt 
+ EinwilligungErteilt 
+ EinwilligungWiderrufen 
+ Datenbankanforderungen 
+ Kundentabelle 
+ Die Kundendatenbank muss folgende Felder unterstützen: 
+ | Feldname                    |
 | --------------------------- |
 | Kundennummer                |
 | Vorname                     |
@@ -2680,15 +2671,15 @@
 | Kundenstatus                |
 | Einwilligungsstatus         |
 | Registrierungsdatum         |
-| LetztesAktualisierungsdatum |
-## Pflichtfelder
-Folgende Felder müssen verpflichtend sein:
-* Kundennummer
-* Vorname
-* Nachname
-* E-Mail-Adresse
-## Datenbankregeln
-* Kundennummern müssen eindeutig sein.</t>
+| LetztesAktualisierungsdatum | 
+ Pflichtfelder 
+ Folgende Felder müssen verpflichtend sein: 
+ Kundennummer 
+ Vorname 
+ Nachname 
+ E-Mail-Adresse 
+ Datenbankregeln 
+ Kundennummern müssen eindeutig sein.</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -2698,14 +2689,14 @@
       </c>
       <c r="E52" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.8403</t>
+          <t>fasttext/0.8722</t>
         </is>
       </c>
       <c r="F52" s="12" t="n">
-        <v>6130</v>
+        <v>6104</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>6928</v>
+        <v>6902</v>
       </c>
     </row>
     <row r="53">
@@ -2720,7 +2711,7 @@
       <c r="C53" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* E-Mail-Adressen dürfen nicht doppelt vergeben werden.</t>
+ E-Mail-Adressen dürfen nicht doppelt vergeben werden.</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
@@ -2734,10 +2725,10 @@
         </is>
       </c>
       <c r="F53" s="9" t="n">
-        <v>6928</v>
+        <v>6903</v>
       </c>
       <c r="G53" s="10" t="n">
-        <v>6984</v>
+        <v>6958</v>
       </c>
     </row>
     <row r="54">
@@ -2752,7 +2743,7 @@
       <c r="C54" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Fremdschlüsselbeziehungen müssen konsistent gehalten werden.</t>
+ Fremdschlüsselbeziehungen müssen konsistent gehalten werden.</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
@@ -2766,10 +2757,10 @@
         </is>
       </c>
       <c r="F54" s="12" t="n">
-        <v>6984</v>
+        <v>6959</v>
       </c>
       <c r="G54" s="13" t="n">
-        <v>7047</v>
+        <v>7021</v>
       </c>
     </row>
     <row r="55">
@@ -2784,7 +2775,7 @@
       <c r="C55" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Soft Deletes shall be supported.</t>
+ Soft Deletes shall be supported.</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
@@ -2798,10 +2789,10 @@
         </is>
       </c>
       <c r="F55" s="9" t="n">
-        <v>7047</v>
+        <v>7022</v>
       </c>
       <c r="G55" s="10" t="n">
-        <v>7082</v>
+        <v>7056</v>
       </c>
     </row>
     <row r="56">
@@ -2816,7 +2807,7 @@
       <c r="C56" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Historische Daten dürfen nicht überschrieben werden.</t>
+ Historische Daten dürfen nicht überschrieben werden.</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -2830,10 +2821,10 @@
         </is>
       </c>
       <c r="F56" s="12" t="n">
-        <v>7082</v>
+        <v>7057</v>
       </c>
       <c r="G56" s="13" t="n">
-        <v>7137</v>
+        <v>7111</v>
       </c>
     </row>
     <row r="57">
@@ -2848,28 +2839,27 @@
       <c r="C57" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# API-Anforderungen
-## Kunde erstellen
-### Endpunkt
-POST /api/kunde/anlegen
-### Anfragefelder
-* Kundennummer
-* Vorname
-* Nachname
-* E-Mail-Adresse
-* Telefonnummer
-* Geburtsdatum
-### Erfolgreiche Antwort
-HTTP Status 201
-### Fehlerbehandlung
-* HTTP 400 – Ungültige Anfrage
-* HTTP 401 – Nicht autorisiert
-* HTTP 403 – Zugriff verweigert
-* HTTP 404 – Ressource nicht gefunden
-* HTTP 409 – Konflikt
-* HTTP 500 – Interner Serverfehler
-Validation errors shall contain detailed descriptions explaining the cause of the failure.</t>
+ API-Anforderungen 
+ Kunde erstellen 
+ Endpunkt 
+ POST /api/kunde/anlegen 
+ Anfragefelder 
+ Kundennummer 
+ Vorname 
+ Nachname 
+ E-Mail-Adresse 
+ Telefonnummer 
+ Geburtsdatum 
+ Erfolgreiche Antwort 
+ HTTP Status 201 
+ Fehlerbehandlung 
+ HTTP 400 – Ungültige Anfrage 
+ HTTP 401 – Nicht autorisiert 
+ HTTP 403 – Zugriff verweigert 
+ HTTP 404 – Ressource nicht gefunden 
+ HTTP 409 – Konflikt 
+ HTTP 500 – Interner Serverfehler 
+ Validation errors shall contain detailed descriptions explaining the cause of the failure.</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
@@ -2879,14 +2869,14 @@
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.5909</t>
+          <t>fasttext/0.6856</t>
         </is>
       </c>
       <c r="F57" s="9" t="n">
-        <v>7137</v>
+        <v>7112</v>
       </c>
       <c r="G57" s="10" t="n">
-        <v>7673</v>
+        <v>7640</v>
       </c>
     </row>
     <row r="58">
@@ -2901,9 +2891,8 @@
       <c r="C58" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# Benutzeroberflächenanforderungen
-The application shall provide a responsive user interface supporting desktop, tablet, and mobile devices.</t>
+ Benutzeroberflächenanforderungen 
+ The application shall provide a responsive user interface supporting desktop, tablet, and mobile devices.</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -2913,14 +2902,14 @@
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.4872</t>
+          <t>fasttext/0.4230</t>
         </is>
       </c>
       <c r="F58" s="12" t="n">
-        <v>7673</v>
+        <v>7641</v>
       </c>
       <c r="G58" s="13" t="n">
-        <v>7821</v>
+        <v>7785</v>
       </c>
     </row>
     <row r="59">
@@ -2935,23 +2924,23 @@
       <c r="C59" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Registerkarten
-* Dashboard
-* Kunden
-* Verträge
-* Berichte
-* Einstellungen
-* Compliance
-* Administration
-## Dashboard
-Das Dashboard muss folgende Informationen anzeigen:
-* Anzahl aktiver Kunden
-* Anzahl neuer Kunden
-* Anzahl offener Vorgänge
-* Anzahl aktiver Verträge
-* Compliance-Kennzahlen
-* Systemstatus
-The dashboard shall refresh data automatically every five minutes.</t>
+ Registerkarten 
+ Dashboard 
+ Kunden 
+ Verträge 
+ Berichte 
+ Einstellungen 
+ Compliance 
+ Administration 
+ Dashboard 
+ Das Dashboard muss folgende Informationen anzeigen: 
+ Anzahl aktiver Kunden 
+ Anzahl neuer Kunden 
+ Anzahl offener Vorgänge 
+ Anzahl aktiver Verträge 
+ Compliance-Kennzahlen 
+ Systemstatus 
+ The dashboard shall refresh data automatically every five minutes.</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
@@ -2961,14 +2950,14 @@
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.8575</t>
+          <t>fasttext/0.8788</t>
         </is>
       </c>
       <c r="F59" s="9" t="n">
-        <v>7821</v>
+        <v>7786</v>
       </c>
       <c r="G59" s="10" t="n">
-        <v>8203</v>
+        <v>8171</v>
       </c>
     </row>
     <row r="60">
@@ -2983,28 +2972,26 @@
       <c r="C60" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# Feldbezeichnungen
-## Kundendaten
-* Kundenname
-* Kundennummer
-* Kundenstatus
-* Vertragsstatus
-* Genehmigungsstatus
-* Vertragsbeginn
-* Vertragsende
-* E-Mail-Adresse
-* Telefonnummer
-* Geburtsdatum
-## Compliance-Daten
-* Einwilligungsstatus
-* Einwilligungsdatum
-* Herkunftssystem
-* Prüfstatus
-* Datenschutzklassifizierung
----
-# Fehlerbehandlung
-Das System muss unerwartete Fehler kontrolliert behandeln.</t>
+ Feldbezeichnungen 
+ Kundendaten 
+ Kundenname 
+ Kundennummer 
+ Kundenstatus 
+ Vertragsstatus 
+ Genehmigungsstatus 
+ Vertragsbeginn 
+ Vertragsende 
+ E-Mail-Adresse 
+ Telefonnummer 
+ Geburtsdatum 
+ Compliance-Daten 
+ Einwilligungsstatus 
+ Einwilligungsdatum 
+ Herkunftssystem 
+ Prüfstatus 
+ Datenschutzklassifizierung 
+ Fehlerbehandlung 
+ Das System muss unerwartete Fehler kontrolliert behandeln.</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -3014,14 +3001,14 @@
       </c>
       <c r="E60" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.8908</t>
+          <t>fasttext/0.9459</t>
         </is>
       </c>
       <c r="F60" s="12" t="n">
-        <v>8203</v>
+        <v>8172</v>
       </c>
       <c r="G60" s="13" t="n">
-        <v>8617</v>
+        <v>8580</v>
       </c>
     </row>
     <row r="61">
@@ -3036,8 +3023,8 @@
       <c r="C61" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Fehlermeldungen
-* Fehler 401: Nicht autorisiert.</t>
+ Fehlermeldungen 
+ Fehler 401: Nicht autorisiert.</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
@@ -3047,14 +3034,14 @@
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.8361</t>
+          <t>fasttext/0.8907</t>
         </is>
       </c>
       <c r="F61" s="9" t="n">
-        <v>8617</v>
+        <v>8581</v>
       </c>
       <c r="G61" s="10" t="n">
-        <v>8671</v>
+        <v>8633</v>
       </c>
     </row>
     <row r="62">
@@ -3069,7 +3056,7 @@
       <c r="C62" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Fehler 403: Zugriff verweigert.</t>
+ Fehler 403: Zugriff verweigert.</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
@@ -3083,10 +3070,10 @@
         </is>
       </c>
       <c r="F62" s="12" t="n">
-        <v>8671</v>
+        <v>8634</v>
       </c>
       <c r="G62" s="13" t="n">
-        <v>8705</v>
+        <v>8667</v>
       </c>
     </row>
     <row r="63">
@@ -3101,7 +3088,7 @@
       <c r="C63" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Fehler 404: Datensatz nicht gefunden.</t>
+ Fehler 404: Datensatz nicht gefunden.</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
@@ -3115,10 +3102,10 @@
         </is>
       </c>
       <c r="F63" s="9" t="n">
-        <v>8705</v>
+        <v>8668</v>
       </c>
       <c r="G63" s="10" t="n">
-        <v>8745</v>
+        <v>8707</v>
       </c>
     </row>
     <row r="64">
@@ -3133,7 +3120,7 @@
       <c r="C64" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Fehler 409: Datensatzkonflikt.</t>
+ Fehler 409: Datensatzkonflikt.</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -3147,10 +3134,10 @@
         </is>
       </c>
       <c r="F64" s="12" t="n">
-        <v>8745</v>
+        <v>8708</v>
       </c>
       <c r="G64" s="13" t="n">
-        <v>8778</v>
+        <v>8740</v>
       </c>
     </row>
     <row r="65">
@@ -3165,7 +3152,7 @@
       <c r="C65" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Fehler 422: Validierungsfehler.</t>
+ Fehler 422: Validierungsfehler.</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -3179,10 +3166,10 @@
         </is>
       </c>
       <c r="F65" s="9" t="n">
-        <v>8778</v>
+        <v>8741</v>
       </c>
       <c r="G65" s="10" t="n">
-        <v>8812</v>
+        <v>8774</v>
       </c>
     </row>
     <row r="66">
@@ -3197,7 +3184,7 @@
       <c r="C66" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-* Fehler 500: Interner Serverfehler.</t>
+ Fehler 500: Interner Serverfehler.</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
@@ -3211,10 +3198,10 @@
         </is>
       </c>
       <c r="F66" s="12" t="n">
-        <v>8812</v>
+        <v>8775</v>
       </c>
       <c r="G66" s="13" t="n">
-        <v>8849</v>
+        <v>8811</v>
       </c>
     </row>
     <row r="67">
@@ -3229,7 +3216,7 @@
       <c r="C67" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-English equivalents shall be available when the user interface language is set to English.</t>
+ English equivalents shall be available when the user interface language is set to English.</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
@@ -3243,10 +3230,10 @@
         </is>
       </c>
       <c r="F67" s="9" t="n">
-        <v>8849</v>
+        <v>8812</v>
       </c>
       <c r="G67" s="10" t="n">
-        <v>8941</v>
+        <v>8906</v>
       </c>
     </row>
     <row r="68">
@@ -3261,9 +3248,8 @@
       <c r="C68" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# Protokollierungsanforderungen
-Alle kritischen Geschäftsoperationen müssen protokolliert werden.</t>
+ Protokollierungsanforderungen 
+ Alle kritischen Geschäftsoperationen müssen protokolliert werden.</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -3273,14 +3259,14 @@
       </c>
       <c r="E68" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.9027</t>
+          <t>fasttext/0.9528</t>
         </is>
       </c>
       <c r="F68" s="12" t="n">
-        <v>8941</v>
+        <v>8907</v>
       </c>
       <c r="G68" s="13" t="n">
-        <v>9046</v>
+        <v>9008</v>
       </c>
     </row>
     <row r="69">
@@ -3295,8 +3281,8 @@
       <c r="C69" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Beispielprotokolle
-2026-03-01 08:00:15 INFO Benutzeranmeldung erfolgreich.</t>
+ Beispielprotokolle 
+ 2026-03-01 08:00:15 INFO Benutzeranmeldung erfolgreich.</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
@@ -3306,14 +3292,14 @@
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.9826</t>
+          <t>fasttext/0.9899</t>
         </is>
       </c>
       <c r="F69" s="9" t="n">
-        <v>9046</v>
+        <v>9009</v>
       </c>
       <c r="G69" s="10" t="n">
-        <v>9126</v>
+        <v>9087</v>
       </c>
     </row>
     <row r="70">
@@ -3328,7 +3314,7 @@
       <c r="C70" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-2026-03-01 08:00:18 INFO Benutzer erfolgreich authentifiziert.</t>
+ 2026-03-01 08:00:18 INFO Benutzer erfolgreich authentifiziert.</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -3342,10 +3328,10 @@
         </is>
       </c>
       <c r="F70" s="12" t="n">
-        <v>9126</v>
+        <v>9088</v>
       </c>
       <c r="G70" s="13" t="n">
-        <v>9190</v>
+        <v>9152</v>
       </c>
     </row>
     <row r="71">
@@ -3360,7 +3346,7 @@
       <c r="C71" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-2026-03-01 08:02:30 WARN Kennwort läuft in 5 Tagen ab.</t>
+ 2026-03-01 08:02:30 WARN Kennwort läuft in 5 Tagen ab.</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
@@ -3374,10 +3360,10 @@
         </is>
       </c>
       <c r="F71" s="9" t="n">
-        <v>9190</v>
+        <v>9153</v>
       </c>
       <c r="G71" s="10" t="n">
-        <v>9246</v>
+        <v>9209</v>
       </c>
     </row>
     <row r="72">
@@ -3392,7 +3378,7 @@
       <c r="C72" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-2026-03-01 08:03:20 ERROR Datenbankverbindung fehlgeschlagen.</t>
+ 2026-03-01 08:03:20 ERROR Datenbankverbindung fehlgeschlagen.</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
@@ -3406,10 +3392,10 @@
         </is>
       </c>
       <c r="F72" s="12" t="n">
-        <v>9246</v>
+        <v>9210</v>
       </c>
       <c r="G72" s="13" t="n">
-        <v>9309</v>
+        <v>9273</v>
       </c>
     </row>
     <row r="73">
@@ -3424,7 +3410,7 @@
       <c r="C73" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-2026-03-01 08:03:21 ERROR Kunde konnte nicht gespeichert werden.</t>
+ 2026-03-01 08:03:21 ERROR Kunde konnte nicht gespeichert werden.</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
@@ -3438,10 +3424,10 @@
         </is>
       </c>
       <c r="F73" s="9" t="n">
-        <v>9309</v>
+        <v>9274</v>
       </c>
       <c r="G73" s="10" t="n">
-        <v>9375</v>
+        <v>9340</v>
       </c>
     </row>
     <row r="74">
@@ -3456,7 +3442,7 @@
       <c r="C74" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-The logging framework shall support structured JSON logging for centralized monitoring systems.</t>
+ The logging framework shall support structured JSON logging for centralized monitoring systems.</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
@@ -3470,10 +3456,10 @@
         </is>
       </c>
       <c r="F74" s="12" t="n">
-        <v>9375</v>
+        <v>9341</v>
       </c>
       <c r="G74" s="13" t="n">
-        <v>9472</v>
+        <v>9438</v>
       </c>
     </row>
     <row r="75">
@@ -3488,9 +3474,8 @@
       <c r="C75" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# Datenschutz- und Compliance-Anforderungen
-Gemäß den geltenden Datenschutzbestimmungen dürfen personenbezogene Daten ausschließlich für legitime Geschäftszwecke verarbeitet werden.</t>
+ Datenschutz- und Compliance-Anforderungen 
+ Gemäß den geltenden Datenschutzbestimmungen dürfen personenbezogene Daten ausschließlich für legitime Geschäftszwecke verarbeitet werden.</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
@@ -3500,14 +3485,14 @@
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.8966</t>
+          <t>fasttext/0.9308</t>
         </is>
       </c>
       <c r="F75" s="9" t="n">
-        <v>9472</v>
+        <v>9439</v>
       </c>
       <c r="G75" s="10" t="n">
-        <v>9661</v>
+        <v>9624</v>
       </c>
     </row>
     <row r="76">
@@ -3522,7 +3507,7 @@
       <c r="C76" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-The organization shall implement appropriate technical and organizational safeguards to protect personal information.</t>
+ The organization shall implement appropriate technical and organizational safeguards to protect personal information.</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -3536,10 +3521,10 @@
         </is>
       </c>
       <c r="F76" s="12" t="n">
-        <v>9661</v>
+        <v>9625</v>
       </c>
       <c r="G76" s="13" t="n">
-        <v>9780</v>
+        <v>9744</v>
       </c>
     </row>
     <row r="77">
@@ -3554,14 +3539,14 @@
       <c r="C77" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Sicherheitsanforderungen
-* Verschlüsselung ruhender Daten
-* Verschlüsselung übertragener Daten
-* Rollenbasierte Zugriffskontrolle
-* Multi-Faktor-Authentifizierung
-* Sicherheitsprotokollierung
-* Regelmäßige Sicherheitsüberprüfungen
-Alle Mitarbeiter sind verpflichtet, Datenschutzrichtlinien einzuhalten.</t>
+ Sicherheitsanforderungen 
+ Verschlüsselung ruhender Daten 
+ Verschlüsselung übertragener Daten 
+ Rollenbasierte Zugriffskontrolle 
+ Multi-Faktor-Authentifizierung 
+ Sicherheitsprotokollierung 
+ Regelmäßige Sicherheitsüberprüfungen 
+ Alle Mitarbeiter sind verpflichtet, Datenschutzrichtlinien einzuhalten.</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
@@ -3571,14 +3556,14 @@
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.9336</t>
+          <t>fasttext/0.9401</t>
         </is>
       </c>
       <c r="F77" s="9" t="n">
-        <v>9780</v>
+        <v>9745</v>
       </c>
       <c r="G77" s="10" t="n">
-        <v>10089</v>
+        <v>10055</v>
       </c>
     </row>
     <row r="78">
@@ -3593,7 +3578,7 @@
       <c r="C78" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-Violations shall be reported immediately to the Data Protection Officer.</t>
+ Violations shall be reported immediately to the Data Protection Officer.</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
@@ -3607,10 +3592,10 @@
         </is>
       </c>
       <c r="F78" s="12" t="n">
-        <v>10089</v>
+        <v>10056</v>
       </c>
       <c r="G78" s="13" t="n">
-        <v>10163</v>
+        <v>10130</v>
       </c>
     </row>
     <row r="79">
@@ -3625,9 +3610,8 @@
       <c r="C79" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# Rechtliche Bestimmungen
-Gemäß §14 Absatz 3 dieser Vereinbarung verpflichtet sich der Auftragnehmer, sämtliche vertraulichen Informationen vertraulich zu behandeln.</t>
+ Rechtliche Bestimmungen 
+ Gemäß §14 Absatz 3 dieser Vereinbarung verpflichtet sich der Auftragnehmer, sämtliche vertraulichen Informationen vertraulich zu behandeln.</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
@@ -3637,14 +3621,14 @@
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.9717</t>
+          <t>fasttext/0.9870</t>
         </is>
       </c>
       <c r="F79" s="9" t="n">
-        <v>10163</v>
+        <v>10131</v>
       </c>
       <c r="G79" s="10" t="n">
-        <v>10336</v>
+        <v>10300</v>
       </c>
     </row>
     <row r="80">
@@ -3659,7 +3643,7 @@
       <c r="C80" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-The Contractor shall not disclose confidential information to any third party without prior written authorization.</t>
+ The Contractor shall not disclose confidential information to any third party without prior written authorization.</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -3673,10 +3657,10 @@
         </is>
       </c>
       <c r="F80" s="12" t="n">
-        <v>10336</v>
+        <v>10301</v>
       </c>
       <c r="G80" s="13" t="n">
-        <v>10452</v>
+        <v>10417</v>
       </c>
     </row>
     <row r="81">
@@ -3691,12 +3675,11 @@
       <c r="C81" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# Support-Ticket-Beispiel
-## Ticketnummer
-INC-1001
-## Benutzermeldung
-"Ich kann die Kundendetailseite nicht öffnen."</t>
+ Support-Ticket-Beispiel 
+ Ticketnummer 
+ INC-1001 
+ Benutzermeldung 
+ "Ich kann die Kundendetailseite nicht öffnen."</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
@@ -3706,14 +3689,14 @@
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.9668</t>
+          <t>fasttext/0.9936</t>
         </is>
       </c>
       <c r="F81" s="9" t="n">
-        <v>10452</v>
+        <v>10418</v>
       </c>
       <c r="G81" s="10" t="n">
-        <v>10579</v>
+        <v>10538</v>
       </c>
     </row>
     <row r="82">
@@ -3728,8 +3711,8 @@
       <c r="C82" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Support-Antwort
-"Das Problem wird derzeit untersucht."</t>
+ Support-Antwort 
+ "Das Problem wird derzeit untersucht."</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
@@ -3739,14 +3722,14 @@
       </c>
       <c r="E82" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.9479</t>
+          <t>fasttext/0.9730</t>
         </is>
       </c>
       <c r="F82" s="12" t="n">
-        <v>10579</v>
+        <v>10539</v>
       </c>
       <c r="G82" s="13" t="n">
-        <v>10639</v>
+        <v>10597</v>
       </c>
     </row>
     <row r="83">
@@ -3761,14 +3744,13 @@
       <c r="C83" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-## Status
-In Bearbeitung
----
-# E-Mail-Beispiel
-## Betreff
-Status der Kundendatenmigration
-Sehr geehrtes Team,
-Die Migration wurde erfolgreich abgeschlossen.</t>
+ Status 
+ In Bearbeitung 
+ E-Mail-Beispiel 
+ Betreff 
+ Status der Kundendatenmigration 
+ Sehr geehrtes Team, 
+ Die Migration wurde erfolgreich abgeschlossen.</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
@@ -3778,14 +3760,14 @@
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.9852</t>
+          <t>fasttext/0.9970</t>
         </is>
       </c>
       <c r="F83" s="9" t="n">
-        <v>10639</v>
+        <v>10598</v>
       </c>
       <c r="G83" s="10" t="n">
-        <v>10804</v>
+        <v>10758</v>
       </c>
     </row>
     <row r="84">
@@ -3813,10 +3795,10 @@
         </is>
       </c>
       <c r="F84" s="12" t="n">
-        <v>10805</v>
+        <v>10759</v>
       </c>
       <c r="G84" s="13" t="n">
-        <v>10884</v>
+        <v>10838</v>
       </c>
     </row>
     <row r="85">
@@ -3831,11 +3813,10 @@
       <c r="C85" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-Mit freundlichen Grüßen
-Projektleitung
----
-# Komplexes Szenario
-Obwohl die Datenmigration erfolgreich abgeschlossen wurde und sämtliche Qualitätsprüfungen positiv verlaufen sind, muss das Projektteam weiterhin die Datenqualität überwachen, da einzelne Altsysteme noch nicht vollständig außer Betrieb genommen wurden, while several downstream applications continue synchronizing customer information across regional environments and compliance validation processes remain active.</t>
+ Mit freundlichen Grüßen 
+ Projektleitung 
+ Komplexes Szenario 
+ Obwohl die Datenmigration erfolgreich abgeschlossen wurde und sämtliche Qualitätsprüfungen positiv verlaufen sind, muss das Projektteam weiterhin die Datenqualität überwachen, da einzelne Altsysteme noch nicht vollständig außer Betrieb genommen wurden, while several downstream applications continue synchronizing customer information across regional environments and compliance validation processes remain active.</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
@@ -3845,14 +3826,14 @@
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>fasttext/0.9680</t>
+          <t>fasttext/0.9747</t>
         </is>
       </c>
       <c r="F85" s="9" t="n">
-        <v>10884</v>
+        <v>10839</v>
       </c>
       <c r="G85" s="10" t="n">
-        <v>11368</v>
+        <v>11321</v>
       </c>
     </row>
     <row r="86">
@@ -3867,9 +3848,8 @@
       <c r="C86" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
----
-# Gemischte Technische Aussage
-Die KundenprofilSynchronisierungsEngine verarbeitet eingehende Ereignisse aus mehreren Quellsystemen und aktualisiert die KundenbeziehungsManagementDatenbank, while the AuditComplianceMonitoringService records every transaction for regulatory reporting, operational monitoring, and long-term audit retention purposes.</t>
+ Gemischte Technische Aussage 
+ Die KundenprofilSynchronisierungsEngine verarbeitet eingehende Ereignisse aus mehreren Quellsystemen und aktualisiert die KundenbeziehungsManagementDatenbank, while the AuditComplianceMonitoringService records every transaction for regulatory reporting, operational monitoring, and long-term audit retention purposes.</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
@@ -3879,14 +3859,14 @@
       </c>
       <c r="E86" s="12" t="inlineStr">
         <is>
-          <t>fasttext/0.8091</t>
+          <t>fasttext/0.8464</t>
         </is>
       </c>
       <c r="F86" s="12" t="n">
-        <v>11368</v>
+        <v>11322</v>
       </c>
       <c r="G86" s="13" t="n">
-        <v>11724</v>
+        <v>11674</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(pipeline): consolidate schemas and update core logic
Refactor the pipeline by replacing multiple US-specific schema files with
standardized STRESS and TEST_DATA schemas. Update splitter and
translation service logic, add database connection utility, and
include new markdown reports and updated test results.
</commit_message>
<xml_diff>
--- a/Hybrid_test_report.xlsx
+++ b/Hybrid_test_report.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>79.617 ms</t>
+          <t>59.244 ms</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="I5" s="10" t="n">
-        <v>121918.2281999965</v>
+        <v>104255.0623000134</v>
       </c>
       <c r="J5" s="10" t="inlineStr">
         <is>
@@ -1083,9 +1083,9 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Projektname: Globale Kundenmanagement-Plattform (GKMP) 
- Projektübersicht 
- Die Globale Kundenmanagement-Plattform (GKMP) stellt eine zentrale Lösung für die Verwaltung von Kundeninformationen über verschiedene Regionen, Geschäftsbereiche und regulatorische Zuständigkeiten hinweg bereit.</t>
+          <t>Projektname: Globale Kundenmanagement-Plattform (GKMP)
+Projektübersicht
+Die Globale Kundenmanagement-Plattform (GKMP) stellt eine zentrale Lösung für die Verwaltung von Kundeninformationen über verschiedene Regionen, Geschäftsbereiche und regulatorische Zuständigkeiten hinweg bereit.</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -1102,7 +1102,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6">
@@ -1130,10 +1130,10 @@
         </is>
       </c>
       <c r="F6" s="12" t="n">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="7">
@@ -1148,7 +1148,7 @@
       <c r="C7" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Die Lösung unterstützt deutschsprachige und englischsprachige Benutzer und ermöglicht eine nahtlose Integration mit bestehenden Unternehmensanwendungen.</t>
+Die Lösung unterstützt deutschsprachige und englischsprachige Benutzer und ermöglicht eine nahtlose Integration mit bestehenden Unternehmensanwendungen.</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -1162,10 +1162,10 @@
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>587</v>
+        <v>584</v>
       </c>
     </row>
     <row r="8">
@@ -1193,10 +1193,10 @@
         </is>
       </c>
       <c r="F8" s="12" t="n">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>783</v>
+        <v>780</v>
       </c>
     </row>
     <row r="9">
@@ -1211,7 +1211,7 @@
       <c r="C9" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Das System muss hochverfügbar sein und eine Verarbeitung großer Datenmengen mit minimaler Latenz gewährleisten.</t>
+Das System muss hochverfügbar sein und eine Verarbeitung großer Datenmengen mit minimaler Latenz gewährleisten.</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
@@ -1225,10 +1225,10 @@
         </is>
       </c>
       <c r="F9" s="9" t="n">
-        <v>784</v>
+        <v>780</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>897</v>
+        <v>893</v>
       </c>
     </row>
     <row r="10">
@@ -1256,10 +1256,10 @@
         </is>
       </c>
       <c r="F10" s="12" t="n">
-        <v>898</v>
+        <v>894</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>1021</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="11">
@@ -1274,8 +1274,8 @@
       <c r="C11" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Geschäftlicher Hintergrund 
- Das Unternehmen betreibt derzeit mehrere voneinander unabhängige Anwendungen zur Speicherung von Kundendaten.</t>
+Geschäftlicher Hintergrund
+Das Unternehmen betreibt derzeit mehrere voneinander unabhängige Anwendungen zur Speicherung von Kundendaten.</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -1289,10 +1289,10 @@
         </is>
       </c>
       <c r="F11" s="9" t="n">
-        <v>1022</v>
+        <v>1017</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>1164</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="12">
@@ -1320,10 +1320,10 @@
         </is>
       </c>
       <c r="F12" s="12" t="n">
-        <v>1165</v>
+        <v>1157</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>1284</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="13">
@@ -1338,7 +1338,7 @@
       <c r="C13" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- The new platform aims to establish a single source of truth for customer information and improve operational efficiency across departments.</t>
+The new platform aims to establish a single source of truth for customer information and improve operational efficiency across departments.</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
@@ -1352,10 +1352,10 @@
         </is>
       </c>
       <c r="F13" s="9" t="n">
-        <v>1285</v>
+        <v>1276</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>1426</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="14">
@@ -1370,7 +1370,7 @@
       <c r="C14" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Mehrere Fachabteilungen haben Bedenken hinsichtlich Datenqualität, Berichtsverzögerungen und regulatorischer Compliance geäußert.</t>
+Mehrere Fachabteilungen haben Bedenken hinsichtlich Datenqualität, Berichtsverzögerungen und regulatorischer Compliance geäußert.</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
@@ -1384,10 +1384,10 @@
         </is>
       </c>
       <c r="F14" s="12" t="n">
-        <v>1427</v>
+        <v>1417</v>
       </c>
       <c r="G14" s="13" t="n">
-        <v>1558</v>
+        <v>1548</v>
       </c>
     </row>
     <row r="15">
@@ -1415,10 +1415,10 @@
         </is>
       </c>
       <c r="F15" s="9" t="n">
-        <v>1559</v>
+        <v>1549</v>
       </c>
       <c r="G15" s="10" t="n">
-        <v>1711</v>
+        <v>1701</v>
       </c>
     </row>
     <row r="16">
@@ -1433,23 +1433,23 @@
       <c r="C16" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Geschäftsziele 
- Primäre Ziele 
- Zentralisierung sämtlicher Kundendaten 
- Verbesserung der Datenqualität 
- Reduzierung redundanter Datensätze 
- Einhaltung regulatorischer Anforderungen 
- Unterstützung internationaler Geschäftsprozesse 
- Verbesserung der Such- und Analysefunktionen 
- Secondary Objectives 
- Faster customer onboarding 
- Improved reporting capabilities 
- Enhanced audit traceability 
- Better integration with third-party systems 
- Reduced operational overhead 
- Benutzerrollen 
- Vertriebssachbearbeiter 
- Der Vertriebssachbearbeiter verwaltet Kundenprofile, erstellt Verträge und pflegt Stammdaten.</t>
+Geschäftsziele
+Primäre Ziele
+Zentralisierung sämtlicher Kundendaten
+Verbesserung der Datenqualität
+Reduzierung redundanter Datensätze
+Einhaltung regulatorischer Anforderungen
+Unterstützung internationaler Geschäftsprozesse
+Verbesserung der Such- und Analysefunktionen
+Secondary Objectives
+Faster customer onboarding
+Improved reporting capabilities
+Enhanced audit traceability
+Better integration with third-party systems
+Reduced operational overhead
+Benutzerrollen
+Vertriebssachbearbeiter
+Der Vertriebssachbearbeiter verwaltet Kundenprofile, erstellt Verträge und pflegt Stammdaten.</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
@@ -1463,10 +1463,10 @@
         </is>
       </c>
       <c r="F16" s="12" t="n">
-        <v>1712</v>
+        <v>1701</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>2339</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="17">
@@ -1481,8 +1481,8 @@
       <c r="C17" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Kundendienstmitarbeiter 
- Customer Service Representatives assist customers, update customer information, and resolve support requests.</t>
+Kundendienstmitarbeiter
+Customer Service Representatives assist customers, update customer information, and resolve support requests.</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -1496,10 +1496,10 @@
         </is>
       </c>
       <c r="F17" s="9" t="n">
-        <v>2340</v>
+        <v>2300</v>
       </c>
       <c r="G17" s="10" t="n">
-        <v>2477</v>
+        <v>2436</v>
       </c>
     </row>
     <row r="18">
@@ -1514,8 +1514,8 @@
       <c r="C18" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Compliance-Beauftragter 
- Der Compliance-Beauftragte überwacht regulatorische Anforderungen und prüft Einwilligungsnachweise.</t>
+Compliance-Beauftragter
+Der Compliance-Beauftragte überwacht regulatorische Anforderungen und prüft Einwilligungsnachweise.</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
@@ -1529,10 +1529,10 @@
         </is>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2478</v>
+        <v>2436</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>2605</v>
+        <v>2562</v>
       </c>
     </row>
     <row r="19">
@@ -1547,8 +1547,8 @@
       <c r="C19" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Systemadministrator 
- System Administrators manage configurations, user access, monitoring, and platform maintenance.</t>
+Systemadministrator
+System Administrators manage configurations, user access, monitoring, and platform maintenance.</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
@@ -1562,10 +1562,10 @@
         </is>
       </c>
       <c r="F19" s="9" t="n">
-        <v>2606</v>
+        <v>2562</v>
       </c>
       <c r="G19" s="10" t="n">
-        <v>2725</v>
+        <v>2680</v>
       </c>
     </row>
     <row r="20">
@@ -1580,8 +1580,8 @@
       <c r="C20" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Berichtsanalyst 
- Reporting Analysts generate operational, financial, and compliance reports.</t>
+Berichtsanalyst
+Reporting Analysts generate operational, financial, and compliance reports.</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
@@ -1595,10 +1595,10 @@
         </is>
       </c>
       <c r="F20" s="12" t="n">
-        <v>2726</v>
+        <v>2680</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>2821</v>
+        <v>2774</v>
       </c>
     </row>
     <row r="21">
@@ -1613,9 +1613,9 @@
       <c r="C21" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- User Story US-001 – Kundensuche 
- Beschreibung 
- Als Kundendienstmitarbeiter möchte ich Kunden anhand verschiedener Suchkriterien finden können, damit ich Kundeninformationen schnell abrufen kann.</t>
+User Story US-001 – Kundensuche
+Beschreibung
+Als Kundendienstmitarbeiter möchte ich Kunden anhand verschiedener Suchkriterien finden können, damit ich Kundeninformationen schnell abrufen kann.</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
@@ -1629,10 +1629,10 @@
         </is>
       </c>
       <c r="F21" s="9" t="n">
-        <v>2822</v>
+        <v>2774</v>
       </c>
       <c r="G21" s="10" t="n">
-        <v>3022</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="22">
@@ -1647,7 +1647,7 @@
       <c r="C22" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- The system shall provide advanced search capabilities supporting exact and fuzzy matching.</t>
+The system shall provide advanced search capabilities supporting exact and fuzzy matching.</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
@@ -1661,10 +1661,10 @@
         </is>
       </c>
       <c r="F22" s="12" t="n">
-        <v>3023</v>
+        <v>2970</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>3115</v>
+        <v>3062</v>
       </c>
     </row>
     <row r="23">
@@ -1679,18 +1679,18 @@
       <c r="C23" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Suchkriterien 
- Der Benutzer soll Kunden anhand folgender Felder suchen können: 
- Kundennummer 
- Vorname 
- Nachname 
- E-Mail-Adresse 
- Telefonnummer 
- Geburtsdatum 
- Vertragsnummer 
- Kundenstatus 
- Akzeptanzkriterien 
- Das Feld "Kundennummer" muss durchsuchbar sein.</t>
+Suchkriterien
+Der Benutzer soll Kunden anhand folgender Felder suchen können:
+Kundennummer
+Vorname
+Nachname
+E-Mail-Adresse
+Telefonnummer
+Geburtsdatum
+Vertragsnummer
+Kundenstatus
+Akzeptanzkriterien
+Das Feld "Kundennummer" muss durchsuchbar sein.</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
@@ -1704,10 +1704,10 @@
         </is>
       </c>
       <c r="F23" s="9" t="n">
-        <v>3116</v>
+        <v>3062</v>
       </c>
       <c r="G23" s="10" t="n">
-        <v>3390</v>
+        <v>3319</v>
       </c>
     </row>
     <row r="24">
@@ -1722,7 +1722,7 @@
       <c r="C24" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Das Feld "Nachname" muss unterstützt werden.</t>
+Das Feld "Nachname" muss unterstützt werden.</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -1736,10 +1736,10 @@
         </is>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3391</v>
+        <v>3319</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>3437</v>
+        <v>3365</v>
       </c>
     </row>
     <row r="25">
@@ -1754,7 +1754,7 @@
       <c r="C25" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Das Feld "Vorname" muss unterstützt werden.</t>
+Das Feld "Vorname" muss unterstützt werden.</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
@@ -1768,10 +1768,10 @@
         </is>
       </c>
       <c r="F25" s="9" t="n">
-        <v>3438</v>
+        <v>3365</v>
       </c>
       <c r="G25" s="10" t="n">
-        <v>3483</v>
+        <v>3410</v>
       </c>
     </row>
     <row r="26">
@@ -1786,7 +1786,7 @@
       <c r="C26" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Search results shall be returned within three seconds.</t>
+Search results shall be returned within three seconds.</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -1800,10 +1800,10 @@
         </is>
       </c>
       <c r="F26" s="12" t="n">
-        <v>3484</v>
+        <v>3410</v>
       </c>
       <c r="G26" s="13" t="n">
-        <v>3540</v>
+        <v>3466</v>
       </c>
     </row>
     <row r="27">
@@ -1818,7 +1818,7 @@
       <c r="C27" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Die Trefferliste muss paginiert dargestellt werden.</t>
+Die Trefferliste muss paginiert dargestellt werden.</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
@@ -1832,10 +1832,10 @@
         </is>
       </c>
       <c r="F27" s="9" t="n">
-        <v>3541</v>
+        <v>3466</v>
       </c>
       <c r="G27" s="10" t="n">
-        <v>3594</v>
+        <v>3519</v>
       </c>
     </row>
     <row r="28">
@@ -1850,7 +1850,7 @@
       <c r="C28" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- The system shall support fuzzy search functionality.</t>
+The system shall support fuzzy search functionality.</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1864,10 +1864,10 @@
         </is>
       </c>
       <c r="F28" s="12" t="n">
-        <v>3595</v>
+        <v>3519</v>
       </c>
       <c r="G28" s="13" t="n">
-        <v>3649</v>
+        <v>3573</v>
       </c>
     </row>
     <row r="29">
@@ -1882,7 +1882,7 @@
       <c r="C29" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Die Suche muss Groß- und Kleinschreibung ignorieren.</t>
+Die Suche muss Groß- und Kleinschreibung ignorieren.</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
@@ -1896,10 +1896,10 @@
         </is>
       </c>
       <c r="F29" s="9" t="n">
-        <v>3650</v>
+        <v>3573</v>
       </c>
       <c r="G29" s="10" t="n">
-        <v>3704</v>
+        <v>3627</v>
       </c>
     </row>
     <row r="30">
@@ -1914,7 +1914,7 @@
       <c r="C30" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Search filters shall support multiple simultaneous criteria.</t>
+Search filters shall support multiple simultaneous criteria.</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1928,10 +1928,10 @@
         </is>
       </c>
       <c r="F30" s="12" t="n">
-        <v>3705</v>
+        <v>3627</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>3767</v>
+        <v>3689</v>
       </c>
     </row>
     <row r="31">
@@ -1946,7 +1946,7 @@
       <c r="C31" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Suchergebnisse müssen nach Relevanz sortiert werden können.</t>
+Suchergebnisse müssen nach Relevanz sortiert werden können.</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
@@ -1960,10 +1960,10 @@
         </is>
       </c>
       <c r="F31" s="9" t="n">
-        <v>3768</v>
+        <v>3689</v>
       </c>
       <c r="G31" s="10" t="n">
-        <v>3829</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="32">
@@ -1978,9 +1978,9 @@
       <c r="C32" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- User Story US-002 – Einwilligungsverwaltung 
- Beschreibung 
- Als Compliance-Beauftragter möchte ich sämtliche Kundeneinwilligungen einsehen können, damit regulatorische Anforderungen überprüft werden können.</t>
+User Story US-002 – Einwilligungsverwaltung
+Beschreibung
+Als Compliance-Beauftragter möchte ich sämtliche Kundeneinwilligungen einsehen können, damit regulatorische Anforderungen überprüft werden können.</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -1994,10 +1994,10 @@
         </is>
       </c>
       <c r="F32" s="12" t="n">
-        <v>3830</v>
+        <v>3750</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>4043</v>
+        <v>3957</v>
       </c>
     </row>
     <row r="33">
@@ -2012,14 +2012,14 @@
       <c r="C33" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Funktionale Anforderungen 
- Der Compliance-Beauftragte muss folgende Informationen anzeigen können: 
- Einwilligungsstatus 
- Zeitstempel 
- Herkunftssystem 
- Änderungsverlauf 
- Verantwortlicher Benutzer 
- The system shall preserve historical records for auditing purposes.</t>
+Funktionale Anforderungen
+Der Compliance-Beauftragte muss folgende Informationen anzeigen können:
+Einwilligungsstatus
+Zeitstempel
+Herkunftssystem
+Änderungsverlauf
+Verantwortlicher Benutzer
+The system shall preserve historical records for auditing purposes.</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
@@ -2033,10 +2033,10 @@
         </is>
       </c>
       <c r="F33" s="9" t="n">
-        <v>4044</v>
+        <v>3957</v>
       </c>
       <c r="G33" s="10" t="n">
-        <v>4320</v>
+        <v>4222</v>
       </c>
     </row>
     <row r="34">
@@ -2051,8 +2051,8 @@
       <c r="C34" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Akzeptanzkriterien 
- Einwilligungshistorien dürfen nicht bearbeitet werden.</t>
+Akzeptanzkriterien
+Einwilligungshistorien dürfen nicht bearbeitet werden.</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -2066,10 +2066,10 @@
         </is>
       </c>
       <c r="F34" s="12" t="n">
-        <v>4321</v>
+        <v>4222</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>4400</v>
+        <v>4298</v>
       </c>
     </row>
     <row r="35">
@@ -2084,7 +2084,7 @@
       <c r="C35" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Änderungen müssen revisionssicher gespeichert werden.</t>
+Änderungen müssen revisionssicher gespeichert werden.</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
@@ -2098,10 +2098,10 @@
         </is>
       </c>
       <c r="F35" s="9" t="n">
-        <v>4401</v>
+        <v>4298</v>
       </c>
       <c r="G35" s="10" t="n">
-        <v>4456</v>
+        <v>4353</v>
       </c>
     </row>
     <row r="36">
@@ -2116,7 +2116,7 @@
       <c r="C36" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Auditberichte müssen als PDF und Excel exportierbar sein.</t>
+Auditberichte müssen als PDF und Excel exportierbar sein.</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -2130,10 +2130,10 @@
         </is>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4457</v>
+        <v>4353</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>4516</v>
+        <v>4412</v>
       </c>
     </row>
     <row r="37">
@@ -2148,7 +2148,7 @@
       <c r="C37" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Das System muss sämtliche Zugriffe protokollieren.</t>
+Das System muss sämtliche Zugriffe protokollieren.</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
@@ -2162,10 +2162,10 @@
         </is>
       </c>
       <c r="F37" s="9" t="n">
-        <v>4517</v>
+        <v>4412</v>
       </c>
       <c r="G37" s="10" t="n">
-        <v>4569</v>
+        <v>4464</v>
       </c>
     </row>
     <row r="38">
@@ -2180,7 +2180,7 @@
       <c r="C38" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Historical records shall remain available indefinitely.</t>
+Historical records shall remain available indefinitely.</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -2194,10 +2194,10 @@
         </is>
       </c>
       <c r="F38" s="12" t="n">
-        <v>4570</v>
+        <v>4464</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>4627</v>
+        <v>4521</v>
       </c>
     </row>
     <row r="39">
@@ -2212,7 +2212,7 @@
       <c r="C39" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Jede Änderung muss einem Benutzer zugeordnet werden können.</t>
+Jede Änderung muss einem Benutzer zugeordnet werden können.</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
@@ -2226,10 +2226,10 @@
         </is>
       </c>
       <c r="F39" s="9" t="n">
-        <v>4628</v>
+        <v>4521</v>
       </c>
       <c r="G39" s="10" t="n">
-        <v>4689</v>
+        <v>4582</v>
       </c>
     </row>
     <row r="40">
@@ -2244,9 +2244,9 @@
       <c r="C40" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Technische Architektur 
- Architekturübersicht 
- The application follows a microservice architecture consisting of independently deployable services.</t>
+Technische Architektur
+Architekturübersicht
+The application follows a microservice architecture consisting of independently deployable services.</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
@@ -2260,10 +2260,10 @@
         </is>
       </c>
       <c r="F40" s="12" t="n">
-        <v>4690</v>
+        <v>4582</v>
       </c>
       <c r="G40" s="13" t="n">
-        <v>4844</v>
+        <v>4730</v>
       </c>
     </row>
     <row r="41">
@@ -2278,7 +2278,7 @@
       <c r="C41" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Jeder Service besitzt eine klar definierte Verantwortlichkeit und kommuniziert über standardisierte REST-Schnittstellen.</t>
+Jeder Service besitzt eine klar definierte Verantwortlichkeit und kommuniziert über standardisierte REST-Schnittstellen.</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -2292,10 +2292,10 @@
         </is>
       </c>
       <c r="F41" s="9" t="n">
-        <v>4845</v>
+        <v>4730</v>
       </c>
       <c r="G41" s="10" t="n">
-        <v>4967</v>
+        <v>4852</v>
       </c>
     </row>
     <row r="42">
@@ -2310,8 +2310,8 @@
       <c r="C42" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- API-Gateway 
- Das API-Gateway fungiert als zentraler Einstiegspunkt für sämtliche Client-Anfragen.</t>
+API-Gateway
+Das API-Gateway fungiert als zentraler Einstiegspunkt für sämtliche Client-Anfragen.</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -2325,10 +2325,10 @@
         </is>
       </c>
       <c r="F42" s="12" t="n">
-        <v>4968</v>
+        <v>4852</v>
       </c>
       <c r="G42" s="13" t="n">
-        <v>5068</v>
+        <v>4951</v>
       </c>
     </row>
     <row r="43">
@@ -2343,18 +2343,18 @@
       <c r="C43" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Funktionen: 
- Authentifizierung 
- Autorisierung 
- Routing 
- Lastverteilung 
- API-Protokollierung 
- Authentifizierung 
- Die Authentifizierung erfolgt über: 
- OAuth 2.0 
- OpenID Connect 
- Multi-Faktor-Authentifizierung 
- The system shall support integration with enterprise identity providers.</t>
+Funktionen:
+Authentifizierung
+Autorisierung
+Routing
+Lastverteilung
+API-Protokollierung
+Authentifizierung
+Die Authentifizierung erfolgt über:
+OAuth 2.0
+OpenID Connect
+Multi-Faktor-Authentifizierung
+The system shall support integration with enterprise identity providers.</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
@@ -2368,10 +2368,10 @@
         </is>
       </c>
       <c r="F43" s="9" t="n">
-        <v>5069</v>
+        <v>4951</v>
       </c>
       <c r="G43" s="10" t="n">
-        <v>5370</v>
+        <v>5233</v>
       </c>
     </row>
     <row r="44">
@@ -2386,9 +2386,9 @@
       <c r="C44" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Kerndienste 
- Kundenservice 
- Verwaltung von Kundenstammdaten und Kundenbeziehungen.</t>
+Kerndienste
+Kundenservice
+Verwaltung von Kundenstammdaten und Kundenbeziehungen.</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
@@ -2402,10 +2402,10 @@
         </is>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5371</v>
+        <v>5233</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>5459</v>
+        <v>5317</v>
       </c>
     </row>
     <row r="45">
@@ -2420,8 +2420,8 @@
       <c r="C45" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Vertragsservice 
- Verwaltung sämtlicher Vertragsinformationen.</t>
+Vertragsservice
+Verwaltung sämtlicher Vertragsinformationen.</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
@@ -2435,10 +2435,10 @@
         </is>
       </c>
       <c r="F45" s="9" t="n">
-        <v>5460</v>
+        <v>5317</v>
       </c>
       <c r="G45" s="10" t="n">
-        <v>5524</v>
+        <v>5380</v>
       </c>
     </row>
     <row r="46">
@@ -2453,8 +2453,8 @@
       <c r="C46" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Benachrichtigungsservice 
- Versand von E-Mails, SMS-Nachrichten und Systembenachrichtigungen.</t>
+Benachrichtigungsservice
+Versand von E-Mails, SMS-Nachrichten und Systembenachrichtigungen.</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
@@ -2468,10 +2468,10 @@
         </is>
       </c>
       <c r="F46" s="12" t="n">
-        <v>5525</v>
+        <v>5380</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>5620</v>
+        <v>5474</v>
       </c>
     </row>
     <row r="47">
@@ -2486,8 +2486,8 @@
       <c r="C47" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Audit-Service 
- Speicherung aller revisionsrelevanten Ereignisse.</t>
+Audit-Service
+Speicherung aller revisionsrelevanten Ereignisse.</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
@@ -2501,10 +2501,10 @@
         </is>
       </c>
       <c r="F47" s="9" t="n">
-        <v>5621</v>
+        <v>5474</v>
       </c>
       <c r="G47" s="10" t="n">
-        <v>5688</v>
+        <v>5540</v>
       </c>
     </row>
     <row r="48">
@@ -2519,8 +2519,8 @@
       <c r="C48" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Berichtsservice 
- Generierung operativer und regulatorischer Berichte.</t>
+Berichtsservice
+Generierung operativer und regulatorischer Berichte.</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
@@ -2534,10 +2534,10 @@
         </is>
       </c>
       <c r="F48" s="12" t="n">
-        <v>5689</v>
+        <v>5540</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>5761</v>
+        <v>5611</v>
       </c>
     </row>
     <row r="49">
@@ -2552,8 +2552,8 @@
       <c r="C49" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Integrationsservice 
- The Integration Service shall synchronize information with external systems.</t>
+Integrationsservice
+The Integration Service shall synchronize information with external systems.</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
@@ -2567,10 +2567,10 @@
         </is>
       </c>
       <c r="F49" s="9" t="n">
-        <v>5762</v>
+        <v>5611</v>
       </c>
       <c r="G49" s="10" t="n">
-        <v>5862</v>
+        <v>5710</v>
       </c>
     </row>
     <row r="50">
@@ -2585,8 +2585,8 @@
       <c r="C50" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Compliance-Service 
- Der Compliance-Service überwacht regulatorische Anforderungen und Datenschutzrichtlinien.</t>
+Compliance-Service
+Der Compliance-Service überwacht regulatorische Anforderungen und Datenschutzrichtlinien.</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -2600,10 +2600,10 @@
         </is>
       </c>
       <c r="F50" s="12" t="n">
-        <v>5863</v>
+        <v>5710</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>5975</v>
+        <v>5821</v>
       </c>
     </row>
     <row r="51">
@@ -2618,8 +2618,8 @@
       <c r="C51" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Ereignisgesteuerte Kommunikation 
- Die Plattform verwendet Apache Kafka für die asynchrone Kommunikation zwischen Services.</t>
+Ereignisgesteuerte Kommunikation
+Die Plattform verwendet Apache Kafka für die asynchrone Kommunikation zwischen Services.</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
@@ -2633,10 +2633,10 @@
         </is>
       </c>
       <c r="F51" s="9" t="n">
-        <v>5976</v>
+        <v>5821</v>
       </c>
       <c r="G51" s="10" t="n">
-        <v>6103</v>
+        <v>5945</v>
       </c>
     </row>
     <row r="52">
@@ -2651,35 +2651,35 @@
       <c r="C52" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Examples of business events: 
- KundeErstellt 
- KundeAktualisiert 
- VertragAngelegt 
- EinwilligungErteilt 
- EinwilligungWiderrufen 
- Datenbankanforderungen 
- Kundentabelle 
- Die Kundendatenbank muss folgende Felder unterstützen: 
- | Feldname                    |
+Examples of business events:
+KundeErstellt
+KundeAktualisiert
+VertragAngelegt
+EinwilligungErteilt
+EinwilligungWiderrufen
+Datenbankanforderungen
+Kundentabelle
+Die Kundendatenbank muss folgende Felder unterstützen:
+| Feldname |
 | --------------------------- |
-| Kundennummer                |
-| Vorname                     |
-| Nachname                    |
-| Geburtsdatum                |
-| E-Mail-Adresse              |
-| Telefonnummer               |
-| Kundenstatus                |
-| Einwilligungsstatus         |
-| Registrierungsdatum         |
-| LetztesAktualisierungsdatum | 
- Pflichtfelder 
- Folgende Felder müssen verpflichtend sein: 
- Kundennummer 
- Vorname 
- Nachname 
- E-Mail-Adresse 
- Datenbankregeln 
- Kundennummern müssen eindeutig sein.</t>
+| Kundennummer |
+| Vorname |
+| Nachname |
+| Geburtsdatum |
+| E-Mail-Adresse |
+| Telefonnummer |
+| Kundenstatus |
+| Einwilligungsstatus |
+| Registrierungsdatum |
+| LetztesAktualisierungsdatum |
+Pflichtfelder
+Folgende Felder müssen verpflichtend sein:
+Kundennummer
+Vorname
+Nachname
+E-Mail-Adresse
+Datenbankregeln
+Kundennummern müssen eindeutig sein.</t>
         </is>
       </c>
       <c r="D52" s="12" t="inlineStr">
@@ -2693,10 +2693,10 @@
         </is>
       </c>
       <c r="F52" s="12" t="n">
-        <v>6104</v>
+        <v>5945</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>6902</v>
+        <v>6568</v>
       </c>
     </row>
     <row r="53">
@@ -2711,7 +2711,7 @@
       <c r="C53" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- E-Mail-Adressen dürfen nicht doppelt vergeben werden.</t>
+E-Mail-Adressen dürfen nicht doppelt vergeben werden.</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
@@ -2725,10 +2725,10 @@
         </is>
       </c>
       <c r="F53" s="9" t="n">
-        <v>6903</v>
+        <v>6568</v>
       </c>
       <c r="G53" s="10" t="n">
-        <v>6958</v>
+        <v>6623</v>
       </c>
     </row>
     <row r="54">
@@ -2743,7 +2743,7 @@
       <c r="C54" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Fremdschlüsselbeziehungen müssen konsistent gehalten werden.</t>
+Fremdschlüsselbeziehungen müssen konsistent gehalten werden.</t>
         </is>
       </c>
       <c r="D54" s="12" t="inlineStr">
@@ -2757,10 +2757,10 @@
         </is>
       </c>
       <c r="F54" s="12" t="n">
-        <v>6959</v>
+        <v>6623</v>
       </c>
       <c r="G54" s="13" t="n">
-        <v>7021</v>
+        <v>6685</v>
       </c>
     </row>
     <row r="55">
@@ -2775,7 +2775,7 @@
       <c r="C55" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Soft Deletes shall be supported.</t>
+Soft Deletes shall be supported.</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
@@ -2789,10 +2789,10 @@
         </is>
       </c>
       <c r="F55" s="9" t="n">
-        <v>7022</v>
+        <v>6685</v>
       </c>
       <c r="G55" s="10" t="n">
-        <v>7056</v>
+        <v>6719</v>
       </c>
     </row>
     <row r="56">
@@ -2807,7 +2807,7 @@
       <c r="C56" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Historische Daten dürfen nicht überschrieben werden.</t>
+Historische Daten dürfen nicht überschrieben werden.</t>
         </is>
       </c>
       <c r="D56" s="12" t="inlineStr">
@@ -2821,10 +2821,10 @@
         </is>
       </c>
       <c r="F56" s="12" t="n">
-        <v>7057</v>
+        <v>6719</v>
       </c>
       <c r="G56" s="13" t="n">
-        <v>7111</v>
+        <v>6773</v>
       </c>
     </row>
     <row r="57">
@@ -2839,27 +2839,27 @@
       <c r="C57" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- API-Anforderungen 
- Kunde erstellen 
- Endpunkt 
- POST /api/kunde/anlegen 
- Anfragefelder 
- Kundennummer 
- Vorname 
- Nachname 
- E-Mail-Adresse 
- Telefonnummer 
- Geburtsdatum 
- Erfolgreiche Antwort 
- HTTP Status 201 
- Fehlerbehandlung 
- HTTP 400 – Ungültige Anfrage 
- HTTP 401 – Nicht autorisiert 
- HTTP 403 – Zugriff verweigert 
- HTTP 404 – Ressource nicht gefunden 
- HTTP 409 – Konflikt 
- HTTP 500 – Interner Serverfehler 
- Validation errors shall contain detailed descriptions explaining the cause of the failure.</t>
+API-Anforderungen
+Kunde erstellen
+Endpunkt
+POST /api/kunde/anlegen
+Anfragefelder
+Kundennummer
+Vorname
+Nachname
+E-Mail-Adresse
+Telefonnummer
+Geburtsdatum
+Erfolgreiche Antwort
+HTTP Status 201
+Fehlerbehandlung
+HTTP 400 – Ungültige Anfrage
+HTTP 401 – Nicht autorisiert
+HTTP 403 – Zugriff verweigert
+HTTP 404 – Ressource nicht gefunden
+HTTP 409 – Konflikt
+HTTP 500 – Interner Serverfehler
+Validation errors shall contain detailed descriptions explaining the cause of the failure.</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
@@ -2873,10 +2873,10 @@
         </is>
       </c>
       <c r="F57" s="9" t="n">
-        <v>7112</v>
+        <v>6773</v>
       </c>
       <c r="G57" s="10" t="n">
-        <v>7640</v>
+        <v>7269</v>
       </c>
     </row>
     <row r="58">
@@ -2891,8 +2891,8 @@
       <c r="C58" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Benutzeroberflächenanforderungen 
- The application shall provide a responsive user interface supporting desktop, tablet, and mobile devices.</t>
+Benutzeroberflächenanforderungen
+The application shall provide a responsive user interface supporting desktop, tablet, and mobile devices.</t>
         </is>
       </c>
       <c r="D58" s="12" t="inlineStr">
@@ -2906,10 +2906,10 @@
         </is>
       </c>
       <c r="F58" s="12" t="n">
-        <v>7641</v>
+        <v>7269</v>
       </c>
       <c r="G58" s="13" t="n">
-        <v>7785</v>
+        <v>7410</v>
       </c>
     </row>
     <row r="59">
@@ -2924,23 +2924,23 @@
       <c r="C59" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Registerkarten 
- Dashboard 
- Kunden 
- Verträge 
- Berichte 
- Einstellungen 
- Compliance 
- Administration 
- Dashboard 
- Das Dashboard muss folgende Informationen anzeigen: 
- Anzahl aktiver Kunden 
- Anzahl neuer Kunden 
- Anzahl offener Vorgänge 
- Anzahl aktiver Verträge 
- Compliance-Kennzahlen 
- Systemstatus 
- The dashboard shall refresh data automatically every five minutes.</t>
+Registerkarten
+Dashboard
+Kunden
+Verträge
+Berichte
+Einstellungen
+Compliance
+Administration
+Dashboard
+Das Dashboard muss folgende Informationen anzeigen:
+Anzahl aktiver Kunden
+Anzahl neuer Kunden
+Anzahl offener Vorgänge
+Anzahl aktiver Verträge
+Compliance-Kennzahlen
+Systemstatus
+The dashboard shall refresh data automatically every five minutes.</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
@@ -2954,10 +2954,10 @@
         </is>
       </c>
       <c r="F59" s="9" t="n">
-        <v>7786</v>
+        <v>7410</v>
       </c>
       <c r="G59" s="10" t="n">
-        <v>8171</v>
+        <v>7771</v>
       </c>
     </row>
     <row r="60">
@@ -2972,26 +2972,26 @@
       <c r="C60" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Feldbezeichnungen 
- Kundendaten 
- Kundenname 
- Kundennummer 
- Kundenstatus 
- Vertragsstatus 
- Genehmigungsstatus 
- Vertragsbeginn 
- Vertragsende 
- E-Mail-Adresse 
- Telefonnummer 
- Geburtsdatum 
- Compliance-Daten 
- Einwilligungsstatus 
- Einwilligungsdatum 
- Herkunftssystem 
- Prüfstatus 
- Datenschutzklassifizierung 
- Fehlerbehandlung 
- Das System muss unerwartete Fehler kontrolliert behandeln.</t>
+Feldbezeichnungen
+Kundendaten
+Kundenname
+Kundennummer
+Kundenstatus
+Vertragsstatus
+Genehmigungsstatus
+Vertragsbeginn
+Vertragsende
+E-Mail-Adresse
+Telefonnummer
+Geburtsdatum
+Compliance-Daten
+Einwilligungsstatus
+Einwilligungsdatum
+Herkunftssystem
+Prüfstatus
+Datenschutzklassifizierung
+Fehlerbehandlung
+Das System muss unerwartete Fehler kontrolliert behandeln.</t>
         </is>
       </c>
       <c r="D60" s="12" t="inlineStr">
@@ -3005,10 +3005,10 @@
         </is>
       </c>
       <c r="F60" s="12" t="n">
-        <v>8172</v>
+        <v>7771</v>
       </c>
       <c r="G60" s="13" t="n">
-        <v>8580</v>
+        <v>8148</v>
       </c>
     </row>
     <row r="61">
@@ -3023,8 +3023,8 @@
       <c r="C61" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Fehlermeldungen 
- Fehler 401: Nicht autorisiert.</t>
+Fehlermeldungen
+Fehler 401: Nicht autorisiert.</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
@@ -3038,10 +3038,10 @@
         </is>
       </c>
       <c r="F61" s="9" t="n">
-        <v>8581</v>
+        <v>8148</v>
       </c>
       <c r="G61" s="10" t="n">
-        <v>8633</v>
+        <v>8197</v>
       </c>
     </row>
     <row r="62">
@@ -3056,7 +3056,7 @@
       <c r="C62" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Fehler 403: Zugriff verweigert.</t>
+Fehler 403: Zugriff verweigert.</t>
         </is>
       </c>
       <c r="D62" s="12" t="inlineStr">
@@ -3070,10 +3070,10 @@
         </is>
       </c>
       <c r="F62" s="12" t="n">
-        <v>8634</v>
+        <v>8197</v>
       </c>
       <c r="G62" s="13" t="n">
-        <v>8667</v>
+        <v>8230</v>
       </c>
     </row>
     <row r="63">
@@ -3088,7 +3088,7 @@
       <c r="C63" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Fehler 404: Datensatz nicht gefunden.</t>
+Fehler 404: Datensatz nicht gefunden.</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
@@ -3102,10 +3102,10 @@
         </is>
       </c>
       <c r="F63" s="9" t="n">
-        <v>8668</v>
+        <v>8230</v>
       </c>
       <c r="G63" s="10" t="n">
-        <v>8707</v>
+        <v>8269</v>
       </c>
     </row>
     <row r="64">
@@ -3120,7 +3120,7 @@
       <c r="C64" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Fehler 409: Datensatzkonflikt.</t>
+Fehler 409: Datensatzkonflikt.</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
@@ -3134,10 +3134,10 @@
         </is>
       </c>
       <c r="F64" s="12" t="n">
-        <v>8708</v>
+        <v>8269</v>
       </c>
       <c r="G64" s="13" t="n">
-        <v>8740</v>
+        <v>8301</v>
       </c>
     </row>
     <row r="65">
@@ -3152,7 +3152,7 @@
       <c r="C65" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Fehler 422: Validierungsfehler.</t>
+Fehler 422: Validierungsfehler.</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -3166,10 +3166,10 @@
         </is>
       </c>
       <c r="F65" s="9" t="n">
-        <v>8741</v>
+        <v>8301</v>
       </c>
       <c r="G65" s="10" t="n">
-        <v>8774</v>
+        <v>8334</v>
       </c>
     </row>
     <row r="66">
@@ -3184,7 +3184,7 @@
       <c r="C66" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Fehler 500: Interner Serverfehler.</t>
+Fehler 500: Interner Serverfehler.</t>
         </is>
       </c>
       <c r="D66" s="12" t="inlineStr">
@@ -3198,10 +3198,10 @@
         </is>
       </c>
       <c r="F66" s="12" t="n">
-        <v>8775</v>
+        <v>8334</v>
       </c>
       <c r="G66" s="13" t="n">
-        <v>8811</v>
+        <v>8370</v>
       </c>
     </row>
     <row r="67">
@@ -3216,7 +3216,7 @@
       <c r="C67" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- English equivalents shall be available when the user interface language is set to English.</t>
+English equivalents shall be available when the user interface language is set to English.</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
@@ -3230,10 +3230,10 @@
         </is>
       </c>
       <c r="F67" s="9" t="n">
-        <v>8812</v>
+        <v>8370</v>
       </c>
       <c r="G67" s="10" t="n">
-        <v>8906</v>
+        <v>8462</v>
       </c>
     </row>
     <row r="68">
@@ -3248,8 +3248,8 @@
       <c r="C68" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Protokollierungsanforderungen 
- Alle kritischen Geschäftsoperationen müssen protokolliert werden.</t>
+Protokollierungsanforderungen
+Alle kritischen Geschäftsoperationen müssen protokolliert werden.</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -3263,10 +3263,10 @@
         </is>
       </c>
       <c r="F68" s="12" t="n">
-        <v>8907</v>
+        <v>8462</v>
       </c>
       <c r="G68" s="13" t="n">
-        <v>9008</v>
+        <v>8560</v>
       </c>
     </row>
     <row r="69">
@@ -3281,8 +3281,8 @@
       <c r="C69" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Beispielprotokolle 
- 2026-03-01 08:00:15 INFO Benutzeranmeldung erfolgreich.</t>
+Beispielprotokolle
+2026-03-01 08:00:15 INFO Benutzeranmeldung erfolgreich.</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
@@ -3296,10 +3296,10 @@
         </is>
       </c>
       <c r="F69" s="9" t="n">
-        <v>9009</v>
+        <v>8560</v>
       </c>
       <c r="G69" s="10" t="n">
-        <v>9087</v>
+        <v>8637</v>
       </c>
     </row>
     <row r="70">
@@ -3314,7 +3314,7 @@
       <c r="C70" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- 2026-03-01 08:00:18 INFO Benutzer erfolgreich authentifiziert.</t>
+2026-03-01 08:00:18 INFO Benutzer erfolgreich authentifiziert.</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -3328,10 +3328,10 @@
         </is>
       </c>
       <c r="F70" s="12" t="n">
-        <v>9088</v>
+        <v>8637</v>
       </c>
       <c r="G70" s="13" t="n">
-        <v>9152</v>
+        <v>8701</v>
       </c>
     </row>
     <row r="71">
@@ -3346,7 +3346,7 @@
       <c r="C71" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- 2026-03-01 08:02:30 WARN Kennwort läuft in 5 Tagen ab.</t>
+2026-03-01 08:02:30 WARN Kennwort läuft in 5 Tagen ab.</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
@@ -3360,10 +3360,10 @@
         </is>
       </c>
       <c r="F71" s="9" t="n">
-        <v>9153</v>
+        <v>8701</v>
       </c>
       <c r="G71" s="10" t="n">
-        <v>9209</v>
+        <v>8757</v>
       </c>
     </row>
     <row r="72">
@@ -3378,7 +3378,7 @@
       <c r="C72" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- 2026-03-01 08:03:20 ERROR Datenbankverbindung fehlgeschlagen.</t>
+2026-03-01 08:03:20 ERROR Datenbankverbindung fehlgeschlagen.</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
@@ -3392,10 +3392,10 @@
         </is>
       </c>
       <c r="F72" s="12" t="n">
-        <v>9210</v>
+        <v>8757</v>
       </c>
       <c r="G72" s="13" t="n">
-        <v>9273</v>
+        <v>8820</v>
       </c>
     </row>
     <row r="73">
@@ -3410,7 +3410,7 @@
       <c r="C73" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- 2026-03-01 08:03:21 ERROR Kunde konnte nicht gespeichert werden.</t>
+2026-03-01 08:03:21 ERROR Kunde konnte nicht gespeichert werden.</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
@@ -3424,10 +3424,10 @@
         </is>
       </c>
       <c r="F73" s="9" t="n">
-        <v>9274</v>
+        <v>8820</v>
       </c>
       <c r="G73" s="10" t="n">
-        <v>9340</v>
+        <v>8886</v>
       </c>
     </row>
     <row r="74">
@@ -3442,7 +3442,7 @@
       <c r="C74" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- The logging framework shall support structured JSON logging for centralized monitoring systems.</t>
+The logging framework shall support structured JSON logging for centralized monitoring systems.</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
@@ -3456,10 +3456,10 @@
         </is>
       </c>
       <c r="F74" s="12" t="n">
-        <v>9341</v>
+        <v>8886</v>
       </c>
       <c r="G74" s="13" t="n">
-        <v>9438</v>
+        <v>8983</v>
       </c>
     </row>
     <row r="75">
@@ -3474,8 +3474,8 @@
       <c r="C75" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Datenschutz- und Compliance-Anforderungen 
- Gemäß den geltenden Datenschutzbestimmungen dürfen personenbezogene Daten ausschließlich für legitime Geschäftszwecke verarbeitet werden.</t>
+Datenschutz- und Compliance-Anforderungen
+Gemäß den geltenden Datenschutzbestimmungen dürfen personenbezogene Daten ausschließlich für legitime Geschäftszwecke verarbeitet werden.</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
@@ -3489,10 +3489,10 @@
         </is>
       </c>
       <c r="F75" s="9" t="n">
-        <v>9439</v>
+        <v>8983</v>
       </c>
       <c r="G75" s="10" t="n">
-        <v>9624</v>
+        <v>9165</v>
       </c>
     </row>
     <row r="76">
@@ -3507,7 +3507,7 @@
       <c r="C76" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- The organization shall implement appropriate technical and organizational safeguards to protect personal information.</t>
+The organization shall implement appropriate technical and organizational safeguards to protect personal information.</t>
         </is>
       </c>
       <c r="D76" s="12" t="inlineStr">
@@ -3521,10 +3521,10 @@
         </is>
       </c>
       <c r="F76" s="12" t="n">
-        <v>9625</v>
+        <v>9165</v>
       </c>
       <c r="G76" s="13" t="n">
-        <v>9744</v>
+        <v>9284</v>
       </c>
     </row>
     <row r="77">
@@ -3539,14 +3539,14 @@
       <c r="C77" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Sicherheitsanforderungen 
- Verschlüsselung ruhender Daten 
- Verschlüsselung übertragener Daten 
- Rollenbasierte Zugriffskontrolle 
- Multi-Faktor-Authentifizierung 
- Sicherheitsprotokollierung 
- Regelmäßige Sicherheitsüberprüfungen 
- Alle Mitarbeiter sind verpflichtet, Datenschutzrichtlinien einzuhalten.</t>
+Sicherheitsanforderungen
+Verschlüsselung ruhender Daten
+Verschlüsselung übertragener Daten
+Rollenbasierte Zugriffskontrolle
+Multi-Faktor-Authentifizierung
+Sicherheitsprotokollierung
+Regelmäßige Sicherheitsüberprüfungen
+Alle Mitarbeiter sind verpflichtet, Datenschutzrichtlinien einzuhalten.</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
@@ -3560,10 +3560,10 @@
         </is>
       </c>
       <c r="F77" s="9" t="n">
-        <v>9745</v>
+        <v>9284</v>
       </c>
       <c r="G77" s="10" t="n">
-        <v>10055</v>
+        <v>9583</v>
       </c>
     </row>
     <row r="78">
@@ -3578,7 +3578,7 @@
       <c r="C78" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Violations shall be reported immediately to the Data Protection Officer.</t>
+Violations shall be reported immediately to the Data Protection Officer.</t>
         </is>
       </c>
       <c r="D78" s="12" t="inlineStr">
@@ -3592,10 +3592,10 @@
         </is>
       </c>
       <c r="F78" s="12" t="n">
-        <v>10056</v>
+        <v>9583</v>
       </c>
       <c r="G78" s="13" t="n">
-        <v>10130</v>
+        <v>9657</v>
       </c>
     </row>
     <row r="79">
@@ -3610,8 +3610,8 @@
       <c r="C79" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Rechtliche Bestimmungen 
- Gemäß §14 Absatz 3 dieser Vereinbarung verpflichtet sich der Auftragnehmer, sämtliche vertraulichen Informationen vertraulich zu behandeln.</t>
+Rechtliche Bestimmungen
+Gemäß §14 Absatz 3 dieser Vereinbarung verpflichtet sich der Auftragnehmer, sämtliche vertraulichen Informationen vertraulich zu behandeln.</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
@@ -3625,10 +3625,10 @@
         </is>
       </c>
       <c r="F79" s="9" t="n">
-        <v>10131</v>
+        <v>9657</v>
       </c>
       <c r="G79" s="10" t="n">
-        <v>10300</v>
+        <v>9823</v>
       </c>
     </row>
     <row r="80">
@@ -3643,7 +3643,7 @@
       <c r="C80" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- The Contractor shall not disclose confidential information to any third party without prior written authorization.</t>
+The Contractor shall not disclose confidential information to any third party without prior written authorization.</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -3657,10 +3657,10 @@
         </is>
       </c>
       <c r="F80" s="12" t="n">
-        <v>10301</v>
+        <v>9823</v>
       </c>
       <c r="G80" s="13" t="n">
-        <v>10417</v>
+        <v>9939</v>
       </c>
     </row>
     <row r="81">
@@ -3675,11 +3675,11 @@
       <c r="C81" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Support-Ticket-Beispiel 
- Ticketnummer 
- INC-1001 
- Benutzermeldung 
- "Ich kann die Kundendetailseite nicht öffnen."</t>
+Support-Ticket-Beispiel
+Ticketnummer
+INC-1001
+Benutzermeldung
+"Ich kann die Kundendetailseite nicht öffnen."</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
@@ -3693,10 +3693,10 @@
         </is>
       </c>
       <c r="F81" s="9" t="n">
-        <v>10418</v>
+        <v>9939</v>
       </c>
       <c r="G81" s="10" t="n">
-        <v>10538</v>
+        <v>10053</v>
       </c>
     </row>
     <row r="82">
@@ -3711,8 +3711,8 @@
       <c r="C82" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Support-Antwort 
- "Das Problem wird derzeit untersucht."</t>
+Support-Antwort
+"Das Problem wird derzeit untersucht."</t>
         </is>
       </c>
       <c r="D82" s="12" t="inlineStr">
@@ -3726,10 +3726,10 @@
         </is>
       </c>
       <c r="F82" s="12" t="n">
-        <v>10539</v>
+        <v>10053</v>
       </c>
       <c r="G82" s="13" t="n">
-        <v>10597</v>
+        <v>10110</v>
       </c>
     </row>
     <row r="83">
@@ -3744,13 +3744,13 @@
       <c r="C83" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Status 
- In Bearbeitung 
- E-Mail-Beispiel 
- Betreff 
- Status der Kundendatenmigration 
- Sehr geehrtes Team, 
- Die Migration wurde erfolgreich abgeschlossen.</t>
+Status
+In Bearbeitung
+E-Mail-Beispiel
+Betreff
+Status der Kundendatenmigration
+Sehr geehrtes Team,
+Die Migration wurde erfolgreich abgeschlossen.</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
@@ -3764,10 +3764,10 @@
         </is>
       </c>
       <c r="F83" s="9" t="n">
-        <v>10598</v>
+        <v>10110</v>
       </c>
       <c r="G83" s="10" t="n">
-        <v>10758</v>
+        <v>10262</v>
       </c>
     </row>
     <row r="84">
@@ -3795,10 +3795,10 @@
         </is>
       </c>
       <c r="F84" s="12" t="n">
-        <v>10759</v>
+        <v>10263</v>
       </c>
       <c r="G84" s="13" t="n">
-        <v>10838</v>
+        <v>10342</v>
       </c>
     </row>
     <row r="85">
@@ -3813,10 +3813,10 @@
       <c r="C85" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Mit freundlichen Grüßen 
- Projektleitung 
- Komplexes Szenario 
- Obwohl die Datenmigration erfolgreich abgeschlossen wurde und sämtliche Qualitätsprüfungen positiv verlaufen sind, muss das Projektteam weiterhin die Datenqualität überwachen, da einzelne Altsysteme noch nicht vollständig außer Betrieb genommen wurden, while several downstream applications continue synchronizing customer information across regional environments and compliance validation processes remain active.</t>
+Mit freundlichen Grüßen
+Projektleitung
+Komplexes Szenario
+Obwohl die Datenmigration erfolgreich abgeschlossen wurde und sämtliche Qualitätsprüfungen positiv verlaufen sind, muss das Projektteam weiterhin die Datenqualität überwachen, da einzelne Altsysteme noch nicht vollständig außer Betrieb genommen wurden, while several downstream applications continue synchronizing customer information across regional environments and compliance validation processes remain active.</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
@@ -3830,10 +3830,10 @@
         </is>
       </c>
       <c r="F85" s="9" t="n">
-        <v>10839</v>
+        <v>10342</v>
       </c>
       <c r="G85" s="10" t="n">
-        <v>11321</v>
+        <v>10819</v>
       </c>
     </row>
     <row r="86">
@@ -3848,8 +3848,8 @@
       <c r="C86" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
- Gemischte Technische Aussage 
- Die KundenprofilSynchronisierungsEngine verarbeitet eingehende Ereignisse aus mehreren Quellsystemen und aktualisiert die KundenbeziehungsManagementDatenbank, while the AuditComplianceMonitoringService records every transaction for regulatory reporting, operational monitoring, and long-term audit retention purposes.</t>
+Gemischte Technische Aussage
+Die KundenprofilSynchronisierungsEngine verarbeitet eingehende Ereignisse aus mehreren Quellsystemen und aktualisiert die KundenbeziehungsManagementDatenbank, while the AuditComplianceMonitoringService records every transaction for regulatory reporting, operational monitoring, and long-term audit retention purposes.</t>
         </is>
       </c>
       <c r="D86" s="12" t="inlineStr">
@@ -3863,10 +3863,10 @@
         </is>
       </c>
       <c r="F86" s="12" t="n">
-        <v>11322</v>
+        <v>10819</v>
       </c>
       <c r="G86" s="13" t="n">
-        <v>11674</v>
+        <v>11168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(config): update gitignore and add schema to kilo config
- add translated_data to .gitignore
- add $schema to .kilo/kilo.json
- add requirements_.txt
</commit_message>
<xml_diff>
--- a/Hybrid_test_report.xlsx
+++ b/Hybrid_test_report.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>59.244 ms</t>
+          <t>77.413 ms</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="I5" s="10" t="n">
-        <v>104255.0623000134</v>
+        <v>69282.69890000047</v>
       </c>
       <c r="J5" s="10" t="inlineStr">
         <is>

</xml_diff>